<commit_message>
docs: cleaner GT answer format in Excel export
- Strip redundant 'table_name:' prefix from structured answers.
- Numbered list (1. 2. 3.) for multi-answer queries.
- Content snippet capped at 150 chars with ellipsis.
- Document vs structured nodes get different formats
  (documents show title ▸ content, structured show content only).

Before: [pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro...
After:  1. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | ...
</commit_message>
<xml_diff>
--- a/eval/data/gt_datasets.xlsx
+++ b/eval/data/gt_datasets.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -887,8 +887,8 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[products:12800001] products:12800001  ▸  products: 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0
-[products:12800007] products:12800007  ▸  products: 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800007 | 69900.0 | 20.0 | 2932 | 204946800.0</t>
+          <t>1. 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0
+2. 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800007 | 69900.0 | 20.0 | 2932 | 204946800.0</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[products:12800004] products:12800004  ▸  products: 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
+          <t>1. 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[products:12800009] products:12800009  ▸  products: 24SS 린넨 와이드 밴딩 슬랙스 | LBL 시즌2025 S/S NO.1 | 24SS | 12800009 | 99900.0 | 20.0 | 4416 | 441158400.0</t>
+          <t>1. 24SS 린넨 와이드 밴딩 슬랙스 | LBL 시즌2025 S/S NO.1 | 24SS | 12800009 | 99900.0 | 20.0 | 4416 | 441158400.0</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[products:12800005] products:12800005  ▸  products: 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0</t>
+          <t>1. 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[colors:1] colors:1  ▸  colors: 소라 | 1</t>
+          <t>1. 소라 | 1</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[colors:4] colors:4  ▸  colors: 네이비 | 4</t>
+          <t>1. 네이비 | 4</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[sizes:2] sizes:2  ▸  sizes: 55 | 2</t>
+          <t>1. 55 | 2</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[reviews:259000003] reviews:259000003  ▸  reviews: 입으면 날씬해 보여요. 핏이 딱 맞아요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000003 | 12800000 | 약간큼</t>
+          <t>1. 입으면 날씬해 보여요. 핏이 딱 맞아요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000003 | 12800000 | 약간큼</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[reviews:259000000] reviews:259000000  ▸  reviews: 세탁해도 줄지 않고 마감이 깔끔해요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 보통이에요 | 착용감 | 아주편해요 | 259000000 | 12800000 | 중</t>
+          <t>1. 세탁해도 줄지 않고 마감이 깔끔해요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 보통이에요 | 착용감 | 아주편해요 | 259000000 | 12800000 | 중</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[reviews:259000004] reviews:259000004  ▸  reviews: 엄마 선물로 구매했는데 너무 좋아하세요. 입으면 편안해요 | 사이즈 | 핏 | 넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000004 | 12800000 | 큼</t>
+          <t>1. 엄마 선물로 구매했는데 너무 좋아하세요. 입으면 편안해요 | 사이즈 | 핏 | 넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000004 | 12800000 | 큼</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[sales_partners:2] sales_partners:2  ▸  sales_partners: 2 | [NEC]패션사업부 | LBL코리아주식회사</t>
+          <t>1. 2 | [NEC]패션사업부 | LBL코리아주식회사</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[sales_channels:1] sales_channels:1  ▸  sales_channels: MC | 1 | EC | MC | OneTV(MC)</t>
+          <t>1. MC | 1 | EC | MC | OneTV(MC)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[broadcasts:1] broadcasts:1  ▸  broadcasts: 1 | 12800000 | 2024-11-15 | 23:00-23:50 | 2024-11-20 | 2024-11-28</t>
+          <t>1. 1 | 12800000 | 2024-11-15 | 23:00-23:50 | 2024-11-20 | 2024-11-28</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[products:12800006] products:12800006  ▸  products: 24FW 데님 A라인 미디 스커트 | LBL 시즌2024 S/S NO.3 | 24FW | 12800006 | 69900.0 | 4314 | 301548600.0</t>
+          <t>1. 24FW 데님 A라인 미디 스커트 | LBL 시즌2024 S/S NO.3 | 24FW | 12800006 | 69900.0 | 4314 | 301548600.0</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[products:12800004] products:12800004  ▸  products: 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
+          <t>1. 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[products:12800009] products:12800009  ▸  products: 24SS 린넨 와이드 밴딩 슬랙스 | LBL 시즌2025 S/S NO.1 | 24SS | 12800009 | 99900.0 | 20.0 | 4416 | 441158400.0</t>
+          <t>1. 24SS 린넨 와이드 밴딩 슬랙스 | LBL 시즌2025 S/S NO.1 | 24SS | 12800009 | 99900.0 | 20.0 | 4416 | 441158400.0</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[products:12800001] products:12800001  ▸  products: 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0</t>
+          <t>1. 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1735,9 +1735,9 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[colors:1] colors:1  ▸  colors: 소라 | 1
-[colors:4] colors:4  ▸  colors: 네이비 | 4
-[colors:5] colors:5  ▸  colors: 블랙 | 5</t>
+          <t>1. 소라 | 1
+2. 네이비 | 4
+3. 블랙 | 5</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1780,9 +1780,9 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0
-[products:12800001] products:12800001  ▸  products: 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0
-[products:12800005] products:12800005  ▸  products: 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0
+2. 24SS 시폰 플리츠 롱 스커트 | LBL 시즌2024 S/S NO.3 | 24SS | 12800001 | 99900.0 | 1862 | 186013800.0
+3. 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[reviews:259000002] reviews:259000002  ▸  reviews: 촉감도 좋고 핏도 라인이 예뻐요 ^^만족합니다 | 사이즈 | 핏 | 타이트해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000002 | 12800000 | 중</t>
+          <t>1. 촉감도 좋고 핏도 라인이 예뻐요 ^^만족합니다 | 사이즈 | 핏 | 타이트해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000002 | 12800000 | 중</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1866,8 +1866,8 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[reviews:259000000] reviews:259000000  ▸  reviews: 세탁해도 줄지 않고 마감이 깔끔해요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 보통이에요 | 착용감 | 아주편해요 | 259000000 | 12800000 | 중
-[reviews:259000004] reviews:259000004  ▸  reviews: 엄마 선물로 구매했는데 너무 좋아하세요. 입으면 편안해요 | 사이즈 | 핏 | 넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000004 | 12800000 | 큼</t>
+          <t>1. 세탁해도 줄지 않고 마감이 깔끔해요 | 사이즈 | 핏 | 약간넉넉해요 | 신축성 | 보통이에요 | 착용감 | 아주편해요 | 259000000 | 12800000 | 중
+2. 엄마 선물로 구매했는데 너무 좋아하세요. 입으면 편안해요 | 사이즈 | 핏 | 넉넉해요 | 신축성 | 잘늘어나요 | 착용감 | 편해요 | 259000004 | 12800000 | 큼</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1909,8 +1909,8 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[products:12800000] products:12800000  ▸  products: 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0
-[products:12800004] products:12800004  ▸  products: 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
+          <t>1. 25SS 실크블렌드 플라워 아플리케 가디건+하프니트 앙상블 | LBL 시즌2024 S/S NO.2 | 25SS | 12800000 | 59900.0 | 10.0 | 2926 | 175267400.0
+2. 24SS 울 캐시미어 브이넥 니트 | LBL 시즌2025 S/S NO.1 | 24SS | 12800004 | 89900.0 | 40.0 | 4547 | 408775300.0</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[sizes:2] sizes:2  ▸  sizes: 55 | 2</t>
+          <t>1. 55 | 2</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[sales_partners:2] sales_partners:2  ▸  sales_partners: 2 | [NEC]패션사업부 | LBL코리아주식회사</t>
+          <t>1. 2 | [NEC]패션사업부 | LBL코리아주식회사</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[broadcasts:1] broadcasts:1  ▸  broadcasts: 1 | 12800000 | 2024-11-15 | 23:00-23:50 | 2024-11-20 | 2024-11-28</t>
+          <t>1. 1 | 12800000 | 2024-11-15 | 23:00-23:50 | 2024-11-20 | 2024-11-28</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2075,8 +2075,8 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[products:12800005] products:12800005  ▸  products: 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0
-[products:12800006] products:12800006  ▸  products: 24FW 데님 A라인 미디 스커트 | LBL 시즌2024 S/S NO.3 | 24FW | 12800006 | 69900.0 | 4314 | 301548600.0</t>
+          <t>1. 24FW 모달 레이스 트리밍 블라우스 | LBL 시즌2024 S/S NO.1 | 24FW | 12800005 | 79900.0 | 20.0 | 3327 | 265827300.0
+2. 24FW 데님 A라인 미디 스커트 | LBL 시즌2024 S/S NO.3 | 24FW | 12800006 | 69900.0 | 4314 | 301548600.0</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2248,8 +2248,8 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[8ff32e537262bfa2] 2020년도_(요약) 2020년 온실가스 감축 및 에너지 절약 업무 추진 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-04-08 16:01:49 &lt;/Document-Metadat
-[d986946925263cee] 2020년도_2020년 온실가스 감축 및 에너지 절약 추진 계획(안) #13  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2011-01-14 09:36:36   수정일: 2020-04-09 11:45:30 &lt;/Document-M</t>
+          <t>1. 2020년도_(요약) 2020년 온실가스 감축 및 에너지 절약 업무 추진 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-04-08 16:01:49 &lt;/Document-Metadata&gt;  ‘20년 온실가스 감축 및 에너지 절약 업무 추…
+2. 2020년도_2020년 온실가스 감축 및 에너지 절약 추진 계획(안) #13  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2011-01-14 09:36:36   수정일: 2020-04-09 11:45:30 &lt;/Document-Metadata&gt;  ❍ 전기 자동차 및 연료전지자동차 구…</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -2295,13 +2295,13 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[9293b657686b140c] 2020년도_200214 (요약) 2020년도 재활힐링승마센터 운영계획(안)ver.6 #14  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: Ryu   작성일: 2020-01-04 13:13:33   수정일: 2020-02-14 11:06:37 &lt;/Document-Metadata&gt;
-[4c2beab48a4fa8ba] 2020년도_200304 (보고)2020년도 재활힐링승마 사업 전략적 홍보방안ver.5 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-05 15:19:27 &lt;/Document-M
-[d3ab6e9ee63de321] 2020년도_200304 2020년도 재활힐링승마 사업 전략적 홍보방안ver.3 #34  ▸  &lt;Document-Metadata&gt;   제목: □    작성자: Ryu   마지막 수정자: Ryu   작성일: 2020-02-20 15:14:45   수정일: 2020-03-04 18:17:25 &lt;/Document-
-[75f6189810773545] 2022년도_재활힐링승마 고도화를 위한 시범과정 운영계획(안) #38  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-03-05 12:48:37   수정일: 2023-04-30 16:21:05 &lt;/Document-Metadata&gt;
-[ae69bf434db74361] 2024년도_재활힐링승마 표준 프로그램 개발연구 시행 계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: □ 2023년 재활힐링승마 시범과정 운영에 따른 사례분석 약식 연구결과   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-05 13:45:52
-[e26613430bc0f1b8] 2020년도_200214 2020년도 재활힐링승마센터 운영계획(안)ver.9 #88  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: Ryu   작성일: 2020-01-04 13:13:33   수정일: 2020-02-14 11:06:08 &lt;/Documen
-[844757da66c84d87] 2024년도_(붙임) 2024년 재활힐링승마 운영 계획(안) #35  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-24 10:15:58   수정일: 2024-02-04 17:57:34 &lt;/Documen</t>
+          <t>1. 2020년도_200214 (요약) 2020년도 재활힐링승마센터 운영계획(안)ver.6 #14  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: Ryu   작성일: 2020-01-04 13:13:33   수정일: 2020-02-14 11:06:37 &lt;/Document-Metadata&gt;  [Image:temp/images/hwp_BIN00…
+2. 2020년도_200304 (보고)2020년도 재활힐링승마 사업 전략적 홍보방안ver.5 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-05 15:19:27 &lt;/Document-Metadata&gt;  ○ 찾아가는 사회공익힐링승마 (상반기…
+3. 2020년도_200304 2020년도 재활힐링승마 사업 전략적 홍보방안ver.3 #34  ▸  &lt;Document-Metadata&gt;   제목: □    작성자: Ryu   마지막 수정자: Ryu   작성일: 2020-02-20 15:14:45   수정일: 2020-03-04 18:17:25 &lt;/Document-Metadata&gt;  예산사항     ○ 총 소요예산 :…
+4. 2022년도_재활힐링승마 고도화를 위한 시범과정 운영계획(안) #38  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-03-05 12:48:37   수정일: 2023-04-30 16:21:05 &lt;/Document-Metadata&gt;  === Extracted Images (Not In…
+5. 2024년도_재활힐링승마 표준 프로그램 개발연구 시행 계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: □ 2023년 재활힐링승마 시범과정 운영에 따른 사례분석 약식 연구결과   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-05 13:45:52   수정일: 2024-06-16 13:48:25 &lt;/Do…
+6. 2020년도_200214 2020년도 재활힐링승마센터 운영계획(안)ver.9 #88  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: Ryu   작성일: 2020-01-04 13:13:33   수정일: 2020-02-14 11:06:08 &lt;/Document-Metadata&gt;  [Image:temp/image…
+7. 2024년도_(붙임) 2024년 재활힐링승마 운영 계획(안) #35  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-24 10:15:58   수정일: 2024-02-04 17:57:34 &lt;/Document-Metadata&gt;  === Extracted Ima…</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -2352,8 +2352,8 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[790f2015dc65b6e1] 2020년도_(붙임#2) 2020년 인재개발 기본계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 인 사 노 무 처   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-02 10:20:11   수정일: 2020-02-27 16:52:55 &lt;/Do
-[33ad8cb9e391ffb3] 2020년도_(붙임#1) 인재개발 기본계획(안) 요약 #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-27 16:38:24 &lt;/Documen</t>
+          <t>1. 2020년도_(붙임#2) 2020년 인재개발 기본계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 인 사 노 무 처   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-02 10:20:11   수정일: 2020-02-27 16:52:55 &lt;/Document-Metadata&gt;  &lt;table borde…
+2. 2020년도_(붙임#1) 인재개발 기본계획(안) 요약 #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-27 16:38:24 &lt;/Document-Metadata&gt;  2020년 인재개발 기본계획(안…</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -2399,10 +2399,10 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[0cf478ddca6e92d5] 2023년도_붙임4 2023년 주요사업 인권영향평가 체크리스트(최종) #29  ▸  &lt;Document-Metadata&gt;   작성자: USER   마지막 수정자: KRA   작성일: 2018-09-04 19:31:17   수정일: 2023-12-21 06:44:31 &lt;/Document-Metadata
-[e507dc22077335c1] 2020년도_별첨_2020년 인권영향평가 결과보고 #14  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2020-11-20 14:17:59   수정일: 2021-05-29 15:46:09 &lt;/Documen
-[dd206af597e56188] 2023년도_붙임1 2023년 인권영향평가 결과보고(최종)★_231222 #11  ▸  &lt;Document-Metadata&gt;   제목: 경영관리처   작성자: KRA   마지막 수정자: KRA   작성일: 2023-12-13 14:18:25   수정일: 2023-12-22 10:01:55 &lt;/Docume
-[005599102a43b8f4] 2023년도_붙임3 2023년 기관운영 인권영향평가 체크리스트(최종) #104  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-09-20 01:25:07   수정일: 2023-12-21 06:47:49 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2023년도_붙임4 2023년 주요사업 인권영향평가 체크리스트(최종) #29  ▸  &lt;Document-Metadata&gt;   작성자: USER   마지막 수정자: KRA   작성일: 2018-09-04 19:31:17   수정일: 2023-12-21 06:44:31 &lt;/Document-Metadata&gt;  [Sheet: 교육, 강습 및 기타 사업] [Ta…
+2. 2020년도_별첨_2020년 인권영향평가 결과보고 #14  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2020-11-20 14:17:59   수정일: 2021-05-29 15:46:09 &lt;/Document-Metadata&gt;  ㅇ (교육 관련 이해관계자 인권…
+3. 2023년도_붙임1 2023년 인권영향평가 결과보고(최종)★_231222 #11  ▸  &lt;Document-Metadata&gt;   제목: 경영관리처   작성자: KRA   마지막 수정자: KRA   작성일: 2023-12-13 14:18:25   수정일: 2023-12-22 10:01:55 &lt;/Document-Metadata&gt;  거 주3일 전환 지속 추진  …
+4. 2023년도_붙임3 2023년 기관운영 인권영향평가 체크리스트(최종) #104  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-09-20 01:25:07   수정일: 2023-12-21 06:47:49 &lt;/Document-Metadata&gt;  [Sheet: 11. 직장 내 인권보호] [Tabl…</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -2450,15 +2450,15 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[2b77cb92e3b2e52e] 2020년도_붙임3. 2020년 총 교배횟수(모든교배내역) #144  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:38:42 &lt;/Document-Metadata&gt;
-[6cdb3f17c1eafe48] 2020년도_붙임2. 2020년 총 교배실적(두수) #111  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:36:12 &lt;/Document-Metadata&gt;
-[bbe40d855e6cc165] 2021년도_경주마 교배 및 번식분야 복지 가이드라인 수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-02 15:44:31 &lt;/Document-M
-[72b1245e55ab96fc] 2021년도_경주마 교배 및 번식분야 복지 가이드라인(안) #17  ▸  &lt;Document-Metadata&gt;   제목: 한국마사회 교배 및 번식 말 복지 가이드라인 초안    작성자: User2007   마지막 수정자: KRA   작성일: 2021-08-07 21:34:58   수정일:
-[57ae80a2b693d18f] 2020년도_붙임4. 2020년 유상교배 수익내역 #6  ▸  &lt;Document-Metadata&gt;   작성자: user   마지막 수정자: KRA   작성일: 2013-10-13 05:56:53   수정일: 2020-12-11 01:28:30 &lt;/Document-Metadata
-[43b8261fe9a4b3ca] 2020년도_@ (결재상신) 2020년 경주마 생산 및 교배지원 결과보고 @ #19  ▸  &lt;Document-Metadata&gt;   제목: 2002. 내륙 민간목장 생산 및 교배지원 결과   작성자: 한국마사회 원당목장팀 대리 임진호   키워드: 
+          <t>1. 2020년도_붙임3. 2020년 총 교배횟수(모든교배내역) #144  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:38:42 &lt;/Document-Metadata&gt;  [Sheet: 2020 총 교배횟수] [Table …
+2. 2020년도_붙임2. 2020년 총 교배실적(두수) #111  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:36:12 &lt;/Document-Metadata&gt;  [Sheet: 2020년 총 교배두수_최종교배기준]…
+3. 2021년도_경주마 교배 및 번식분야 복지 가이드라인 수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-02 15:44:31 &lt;/Document-Metadata&gt;  경주마 교배 및 번식분야 복지 가이드…
+4. 2021년도_경주마 교배 및 번식분야 복지 가이드라인(안) #17  ▸  &lt;Document-Metadata&gt;   제목: 한국마사회 교배 및 번식 말 복지 가이드라인 초안    작성자: User2007   마지막 수정자: KRA   작성일: 2021-08-07 21:34:58   수정일: 2021-12-02 11:22:35 &lt;/Document…
+5. 2020년도_붙임4. 2020년 유상교배 수익내역 #6  ▸  &lt;Document-Metadata&gt;   작성자: user   마지막 수정자: KRA   작성일: 2013-10-13 05:56:53   수정일: 2020-12-11 01:28:30 &lt;/Document-Metadata&gt;  [Sheet: 작업용] [Table Chunk 7…
+6. 2020년도_@ (결재상신) 2020년 경주마 생산 및 교배지원 결과보고 @ #19  ▸  &lt;Document-Metadata&gt;   제목: 2002. 내륙 민간목장 생산 및 교배지원 결과   작성자: 한국마사회 원당목장팀 대리 임진호   키워드: 
     설명: 
-    마지막 수정자: KRA
-[e39b4656a5219700] 2020년도_@ (요약) 2020년 경주마 생산 및 교배지원 결과보고 @ #3  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-12-17 11:13:23 &lt;/Document-Metadat</t>
+    마지막 수정자: KRA   작성일: 2005-08-25 10:09:53   수정…
+7. 2020년도_@ (요약) 2020년 경주마 생산 및 교배지원 결과보고 @ #3  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-12-17 11:13:23 &lt;/Document-Metadata&gt;  두, 민간 1,485두)      ○ 전체 대비…</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -2509,8 +2509,8 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[803aa364d8f1f722] 2021년도_(별첨) 한국마사회 인권침해 구제절차 및 예방활동 매뉴얼(202112) #0  ▸  &lt;Document-Metadata&gt;   제목: 2017   작성자: ROEN11   마지막 수정자: KRA   작성일: 2017-11-20 09:30:38   수정일: 2023-04-13 13:51:00 &lt;/Docu
-[e074f8fc80056924] 2023년도_(별첨) 한국마사회 인권침해 구제절차 및 예방활동 매뉴얼(202112) #0  ▸  &lt;Document-Metadata&gt;   제목: 2017   작성자: ROEN11   마지막 수정자: KRA   작성일: 2017-11-20 09:30:38   수정일: 2023-04-13 13:51:00 &lt;/Docu</t>
+          <t>1. 2021년도_(별첨) 한국마사회 인권침해 구제절차 및 예방활동 매뉴얼(202112) #0  ▸  &lt;Document-Metadata&gt;   제목: 2017   작성자: ROEN11   마지막 수정자: KRA   작성일: 2017-11-20 09:30:38   수정일: 2023-04-13 13:51:00 &lt;/Document-Metadata&gt;  &lt;table border=…
+2. 2023년도_(별첨) 한국마사회 인권침해 구제절차 및 예방활동 매뉴얼(202112) #0  ▸  &lt;Document-Metadata&gt;   제목: 2017   작성자: ROEN11   마지막 수정자: KRA   작성일: 2017-11-20 09:30:38   수정일: 2023-04-13 13:51:00 &lt;/Document-Metadata&gt;  &lt;table border=…</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -2556,10 +2556,10 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[3b6b26357ad2ce21] 2020년도_(요약) 2020년 이용자보호 추진계획 보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-21 13:18:29 &lt;/Document-M
-[24413d0baba3f505] 2020년도_(붙임)'20 이용자보호 현업과제 운영계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제도 확산   작성자: KRA   마지막 수정자: KRA   작성일: 2020-06-12 15:43:26   수정일: 2020-07-25 17:48:38 &lt;/Docume
-[d4d20ca93dfcd728] 2020년도_(본문) 2020년 이용자보호 추진계획 #15  ▸  &lt;Document-Metadata&gt;   제목: 회의자료    작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-19 16:10:55   수정일: 2020-03-21 10:39:32 &lt;/Docume
-[5d0dd8502b5a0cb8] 2020년도_(본문) 20년 이용자보호 액션플랜 수립계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 제목    작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-16 09:57:57   수정일: 2020-02-09 15:46:56 &lt;/Document</t>
+          <t>1. 2020년도_(요약) 2020년 이용자보호 추진계획 보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-21 13:18:29 &lt;/Document-Metadata&gt;  * 세부 추진계획은 과제별로 별도 수…
+2. 2020년도_(붙임)'20 이용자보호 현업과제 운영계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제도 확산   작성자: KRA   마지막 수정자: KRA   작성일: 2020-06-12 15:43:26   수정일: 2020-07-25 17:48:38 &lt;/Document-Metadata&gt;  가. 추진절차  &lt;table …
+3. 2020년도_(본문) 2020년 이용자보호 추진계획 #15  ▸  &lt;Document-Metadata&gt;   제목: 회의자료    작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-19 16:10:55   수정일: 2020-03-21 10:39:32 &lt;/Document-Metadata&gt;  (고객보호부) 과제 총괄 관리…
+4. 2020년도_(본문) 20년 이용자보호 액션플랜 수립계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 제목    작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-16 09:57:57   수정일: 2020-02-09 15:46:56 &lt;/Document-Metadata&gt;  [Image:temp/images…</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -2607,8 +2607,8 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[012dcbe84f52c595] 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Me
-[2df376eb9253a430] 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Me</t>
+          <t>1. 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…
+2. 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -2654,9 +2654,9 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[d13b5751987d7a60] 2021년도_(본문) 사회적가치 실현을 위한 2021년 윤리경영 기본계획(안) #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-02 16:19:40   수정일: 2021-07-15 10:25:51 &lt;/Document-Metadata&gt;
-[d908c9b95b9e082a] 2021년도_(요약) 2021년 윤리경영 기본계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2021-07-15 10:
-[8c423366bc12e4d4] 2023년도_★(결재) 2023년 윤리경영 기본계획(이사회 의견 반영 후)★ #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-06-11 15:07:02   수정일: 2023-07-01 14:03:33 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2021년도_(본문) 사회적가치 실현을 위한 2021년 윤리경영 기본계획(안) #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-02 16:19:40   수정일: 2021-07-15 10:25:51 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+2. 2021년도_(요약) 2021년 윤리경영 기본계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2021-07-15 10:28:48 &lt;/Document-Metadata&gt;  조사…
+3. 2023년도_★(결재) 2023년 윤리경영 기본계획(이사회 의견 반영 후)★ #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-06-11 15:07:02   수정일: 2023-07-01 14:03:33 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -2703,9 +2703,9 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[a4ed66c59a820e40] 2020년도_(붙임#14) 사업별 조직별 예산 계층구조 #78  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-11 08:44:57   수정일: 2020-03-13 01:24:08 &lt;/Document-Metadata&gt;
-[da8efb3618249a33] 2022년도_[붙임2] 2023년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-02-15 02:28:16   수정일: 2023-02-16 04:38:18 &lt;/Document-Metadata&gt;
-[aa6aff98e2caa723] 2023년도_[붙임2] 2024년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-14 07:46:48   수정일: 2024-01-31 07:29:46 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2020년도_(붙임#14) 사업별 조직별 예산 계층구조 #78  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-11 08:44:57   수정일: 2020-03-13 01:24:08 &lt;/Document-Metadata&gt;  [Sheet: 사업별 예산 계층구조] [Table …
+2. 2022년도_[붙임2] 2023년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-02-15 02:28:16   수정일: 2023-02-16 04:38:18 &lt;/Document-Metadata&gt;  [Sheet: 조직별 예산 계층구조] [Table …
+3. 2023년도_[붙임2] 2024년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-14 07:46:48   수정일: 2024-01-31 07:29:46 &lt;/Document-Metadata&gt;  [Sheet: 조직별 예산 계층구조] [Table …</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -2752,10 +2752,10 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[436d43261922a8da] 2020년도_(기재부) 2020년도 예산 및 기금운용계획집행지침 #120  ▸  &lt;Document-Metadata&gt;   제목: ?    작성자: Owner   키워드: 
+          <t>1. 2020년도_(기재부) 2020년도 예산 및 기금운용계획집행지침 #120  ▸  &lt;Document-Metadata&gt;   제목: ?    작성자: Owner   키워드: 
     설명: 
-    마지막 수정자: mafra   작성일: 2005-01-14 10:13:01   수정일: 20
-[4196a8bfffd7ea93] 2024년도_[붙임3] (기재부) 2024년도 예산 및 기금운용계획 집행지침 #282  ▸  &lt;Document-Metadata&gt;   Version Tagetapplication: WORDPROCESSOR   Version Major: 5   Version Minor: 0   Version Micro: 5</t>
+    마지막 수정자: mafra   작성일: 2005-01-14 10:13:01   수정일: 2020-01-08 11:01:36 &lt;/Document-M…
+2. 2024년도_[붙임3] (기재부) 2024년도 예산 및 기금운용계획 집행지침 #282  ▸  &lt;Document-Metadata&gt;   Version Tagetapplication: WORDPROCESSOR   Version Major: 5   Version Minor: 0   Version Micro: 5   Version Buildnumber: 0   Vers…</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -2801,8 +2801,8 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[27325f8e49d559f4] 2020년도_(본문) 2020년도 내부경영평가제도 개선(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-22 09:53:12 &lt;/Documen
-[06ea8eb0c6498c61] 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-M</t>
+          <t>1. 2020년도_(본문) 2020년도 내부경영평가제도 개선(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-22 09:53:12 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+2. 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-Metadata&gt;  가와 사업성과평가 통합    ◦ (차…</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[36f5479362d3d864] 2020년도_201020 지사 고객입장 및 방역관리 방안(최종) #25  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-10-16 08:23:47   수정일: 2020-10-20 18:44:49 &lt;/Documen</t>
+          <t>1. 2020년도_201020 지사 고객입장 및 방역관리 방안(최종) #25  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-10-16 08:23:47   수정일: 2020-10-20 18:44:49 &lt;/Document-Metadata&gt;  [Image:temp/image…</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -2893,9 +2893,9 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[afd0f60cc9c978c0] 2022년도_붙임 1. 스마트 사무환경 구축 및 망분리 개선 견적서(총괄) #27  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-02 04:07:54   수정일: 2023-08-17 03:33:36 &lt;/Document-Metadata&gt;
-[9d226cce773a4434] 2022년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Documen
-[993ad9a5e29994fc] 2023년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Documen</t>
+          <t>1. 2022년도_붙임 1. 스마트 사무환경 구축 및 망분리 개선 견적서(총괄) #27  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-02 04:07:54   수정일: 2023-08-17 03:33:36 &lt;/Document-Metadata&gt;  [Sheet: 3.2 SSD] [Image:temp…
+2. 2022년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Document-Metadata&gt;  [Image:temp/image…
+3. 2023년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Document-Metadata&gt;  [Image:temp/image…</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2942,10 +2942,10 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[c8ed7811592eac64] 2022년도_(붙임2)재물조사결과내역(전체) #393  ▸  &lt;Document-Metadata&gt;   작성일: 2025-12-05 08:14:00   수정일: 2025-12-05 08:14:00 &lt;/Document-Metadata&gt;  [Page Number: 394]  &lt;tab
-[59854a9e60c7d3ab] 2022년도_(붙임2)재물조사결과내역(전체) #106  ▸  &lt;Document-Metadata&gt;   작성자: KA B &lt;/Document-Metadata&gt;  [Sheet: 전체] [Table Chunk 107/107] | 자산번호 | SAP자산번호 | 자산구분 | 세분류 |
-[6a278de5a7f63982] 2022년도_(붙임1)2022년 정기 재물조사 실시 결과보고 #9  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-23 10:36:27   수정일: 2023-01-19 14:22:42 &lt;/Documen
-[95765c577ef9e336] 2024년도_(붙임1) 2024년 재물조사 시행 결과보고_241227 #15  ▸  &lt;Document-Metadata&gt;   제목: 재물조정   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-12 16:02:40   수정일: 2024-12-27 09:49:24 &lt;/Documen</t>
+          <t>1. 2022년도_(붙임2)재물조사결과내역(전체) #393  ▸  &lt;Document-Metadata&gt;   작성일: 2025-12-05 08:14:00   수정일: 2025-12-05 08:14:00 &lt;/Document-Metadata&gt;  [Page Number: 394]  &lt;table&gt;   &lt;tr&gt;     &lt;th&gt;20220842911…
+2. 2022년도_(붙임2)재물조사결과내역(전체) #106  ▸  &lt;Document-Metadata&gt;   작성자: KA B &lt;/Document-Metadata&gt;  [Sheet: 전체] [Table Chunk 107/107] | 자산번호 | SAP자산번호 | 자산구분 | 세분류 | 본부명 | 자산내역 | 취득일자 | 구매금액 | 단가 …
+3. 2022년도_(붙임1)2022년 정기 재물조사 실시 결과보고 #9  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-23 10:36:27   수정일: 2023-01-19 14:22:42 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+4. 2024년도_(붙임1) 2024년 재물조사 시행 결과보고_241227 #15  ▸  &lt;Document-Metadata&gt;   제목: 재물조정   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-12 16:02:40   수정일: 2024-12-27 09:49:24 &lt;/Document-Metadata&gt;  전 부서    ❍ 조직개편, 인…</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2993,8 +2993,8 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>[e4f72caaf5619284] 2023년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;
-[7d016a8eb300196a] 2024년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2023년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;  [Sheet: 15년도 이하 소형복합기] [Tabl…
+2. 2024년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;  [Sheet: 15년도 이하 소형복합기] [Tabl…</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -3040,8 +3040,8 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>[1dd7a41b6d49067a] 2020년도_붙임_2_2020년 도심승마체험 시행계획(본문, 최종) #55  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-09 13:50:33   수정일: 2020-03-11 10:31:15 &lt;/Document-M
-[68c173524cf22c47] 2020년도_붙임_1_2020년 도심승마체험 시행계획(요약, 최종) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-03-07 18:01:46 &lt;/Document-Metadat</t>
+          <t>1. 2020년도_붙임_2_2020년 도심승마체험 시행계획(본문, 최종) #55  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-09 13:50:33   수정일: 2020-03-11 10:31:15 &lt;/Document-Metadata&gt;  === Extracted Images…
+2. 2020년도_붙임_1_2020년 도심승마체험 시행계획(요약, 최종) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-03-07 18:01:46 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;t…</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -3087,8 +3087,8 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>[a5a7f37b741bdeee] 2020년도_제2차 KPC 개최계획(안) 최종 #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-21 09:21:54   수정일: 2020-08-21 17:42:45 &lt;/Document-Metadata&gt;
-[33640ab36a7a2b8c] 2024년도_2024년 제 2차 KPC 개최 심의 안건 #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-18 12:53:46 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2020년도_제2차 KPC 개최계획(안) 최종 #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-21 09:21:54   수정일: 2020-08-21 17:42:45 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+2. 2024년도_2024년 제 2차 KPC 개최 심의 안건 #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-18 12:53:46 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -3134,26 +3134,26 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>[dd534b8aff2c0b47] 2023년도_(별첨2)말산업 연구사업 과제목록(13-23) #23  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2024-03-30 11:46:30 &lt;/Document-Metadata&gt;
-[858311a17598e098] 2024년도_(별첨2)말산업 연구사업 과제목록(13-23) #23  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2024-03-30 11:46:30 &lt;/Document-Metadata&gt;
-[37d0fe4807f770c9] 2020년도_2020년 말산업 연구사업 추진계획(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2020-05-30 14:55:48 &lt;/Document-M
-[665c95e2452936a4] 2021년도_2021년 말산업 연구사업 추진계획(요약,결재용) #3  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-05-08 09:19:09 &lt;/Documen
-[6498c34e04755c85] 2021년도_[붙임2] 2021년 말산업 분야 기술상용화 연구 추진계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-06-20 11:32:59 &lt;/Documen
-[ca05784c3e5aac4f] 2023년도_2023년 말산업 연구사업 추진계획(요약) #2  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2023-04-05 15:06:47 &lt;/Documen
-[9ef0a8ba81ba8b76] 2024년도_2024년 말산업연구소 주요사업 추진계획(본문)  ▸  2024년도_2024년 말산업연구소 주요사업 추진계획(본문)
-[5751364a07bd6432] 2022년도_(별첨2)말산업연구소 연구과제 목록('13_'22) #22  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2023-04-05 01:26:43 &lt;/Document-Metadata&gt;
-[a327f99bb35ec842] 2020년도_2020년 말산업 연구사업 추진계획(요약) #2  ▸  &lt;Document-Metadata&gt;   작성자: 류성훈   마지막 수정자: KRA   작성일: 2014-07-03 13:36:03   수정일: 2020-05-30 15:39:20 &lt;/Document-Metadata&gt;
-[72abd3a0e6e49e3b] 2020년도_[붙임1] 2020년 말산업 분야 위탁연구과제 추진 계획(안) #7  ▸  &lt;Document-Metadata&gt;   제목: 2016   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-25 11:04:51   수정일: 2020-06-24 16:38:49 &lt;/Documen
-[7391433818c2aa29] 2021년도_2021년 말산업 연구사업 추진계획(안,결재용) #10  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2021-05-09 17:06:29 &lt;/Document-M
-[fd1f3b6cb4f3c808] 2021년도_[붙임1] 2021년 말산업 분야 기술상용화 연구 추진계획(요약) #4  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-06-20 11:32:44 &lt;/Documen
-[69aa111c4c3c9c4e] 2023년도_2023년 말산업 연구사업 변경 및 신규과제 추진계획(요약) #3  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2023-12-21 10:35:31 &lt;/Documen
-[425d5a095aa05d99] 2023년도_2023년 말산업 연구사업 추진계획(본문) #16  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2023-04-05 15:01:17 &lt;/Document-M
-[530eee4771fc7f6a] 2023년도_2023년 말산업연구소 주요사업 추진계획(본문)  ▸  2023년도_2023년 말산업연구소 주요사업 추진계획(본문)
-[3069278768910766] 2023년도_2023년 말산업연구소 주요사업 추진계획(요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2023-03-09 15:45:08 &lt;/Documen
-[dce393b4643910d6] 2023년도_23년_말산업_R&amp;D_연구과제_변경_및 _추진계획(안)) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-12-21 09:45:12 &lt;/Document-M
-[7b6883061d74991f] 2024년도_2024년 말산업 연구사업 추진계획(본문) #25  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2024-03-31 10:52:49 &lt;/Document-M
-[c7acbf436686b08b] 2024년도_2024년 말산업 연구사업 추진계획(요약) #12  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2024-03-31 11:13:34 &lt;/Documen
-[f7f1618283b6dd00] 2024년도_2024년 말산업연구소 주요사업 추진계획(본문)  ▸  2024년도_2024년 말산업연구소 주요사업 추진계획(본문)
+          <t>1. 2023년도_(별첨2)말산업 연구사업 과제목록(13-23) #23  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2024-03-30 11:46:30 &lt;/Document-Metadata&gt;  [Sheet: 분야별] [Table 3] | 계 |…
+2. 2024년도_(별첨2)말산업 연구사업 과제목록(13-23) #23  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2024-03-30 11:46:30 &lt;/Document-Metadata&gt;  [Sheet: 분야별] [Table 3] | 계 |…
+3. 2020년도_2020년 말산업 연구사업 추진계획(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2020-05-30 14:55:48 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+4. 2021년도_2021년 말산업 연구사업 추진계획(요약,결재용) #3  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-05-08 09:19:09 &lt;/Document-Metadata&gt;  * 3번 과제는 제주대와 협업하…
+5. 2021년도_[붙임2] 2021년 말산업 분야 기술상용화 연구 추진계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-06-20 11:32:59 &lt;/Document-Metadata&gt;  4. 소요예산 : 축발기금  &lt;…
+6. 2023년도_2023년 말산업 연구사업 추진계획(요약) #2  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2023-04-05 15:06:47 &lt;/Document-Metadata&gt;  ※ 2022년도 연구사업 7개 …
+7. 2024년도_2024년 말산업연구소 주요사업 추진계획(본문)  ▸  2024년도_2024년 말산업연구소 주요사업 추진계획(본문)
+8. 2022년도_(별첨2)말산업연구소 연구과제 목록('13_'22) #22  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-05 04:00:04   수정일: 2023-04-05 01:26:43 &lt;/Document-Metadata&gt;  [Sheet: 분야별] [Table 3] | 계 |…
+9. 2020년도_2020년 말산업 연구사업 추진계획(요약) #2  ▸  &lt;Document-Metadata&gt;   작성자: 류성훈   마지막 수정자: KRA   작성일: 2014-07-03 13:36:03   수정일: 2020-05-30 15:39:20 &lt;/Document-Metadata&gt;  ※ 민간대상 말산업 기술분야 자율공모(1건) 별도 …
+10. 2020년도_[붙임1] 2020년 말산업 분야 위탁연구과제 추진 계획(안) #7  ▸  &lt;Document-Metadata&gt;   제목: 2016   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-25 11:04:51   수정일: 2020-06-24 16:38:49 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+11. 2021년도_2021년 말산업 연구사업 추진계획(안,결재용) #10  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2021-05-09 17:06:29 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+12. 2021년도_[붙임1] 2021년 말산업 분야 기술상용화 연구 추진계획(요약) #4  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2021-06-20 11:32:44 &lt;/Document-Metadata&gt;  1.gif]         * …
+13. 2023년도_2023년 말산업 연구사업 변경 및 신규과제 추진계획(요약) #3  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2023-12-21 10:35:31 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+14. 2023년도_2023년 말산업 연구사업 추진계획(본문) #16  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2023-04-05 15:01:17 &lt;/Document-Metadata&gt;  자체예산 과제  &lt;table bord…
+15. 2023년도_2023년 말산업연구소 주요사업 추진계획(본문)  ▸  2023년도_2023년 말산업연구소 주요사업 추진계획(본문)
+16. 2023년도_2023년 말산업연구소 주요사업 추진계획(요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2023-03-09 15:45:08 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+17. 2023년도_23년_말산업_R&amp;D_연구과제_변경_및 _추진계획(안)) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-12-21 09:45:12 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+18. 2024년도_2024년 말산업 연구사업 추진계획(본문) #25  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-15 10:56:58   수정일: 2024-03-31 10:52:49 &lt;/Document-Metadata&gt;  (축발기금과제) 축발기금 내 R&amp;D …
+19. 2024년도_2024년 말산업 연구사업 추진계획(요약) #12  ▸  &lt;Document-Metadata&gt;   제목: 운영경과   작성자: Ryu   마지막 수정자: KRA   작성일: 2021-03-10 15:28:13   수정일: 2024-03-31 11:13:34 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+20. 2024년도_2024년 말산업연구소 주요사업 추진계획(본문)  ▸  2024년도_2024년 말산업연구소 주요사업 추진계획(본문)
 ... +2 more</t>
         </is>
       </c>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>[157016074626f25d] 2021년도_(별첨1) 연도별 마주 경제적기준(2007_2021) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-20 01:23:19   수정일: 2021-11-26 04:01:22 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2021년도_(별첨1) 연도별 마주 경제적기준(2007_2021) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-20 01:23:19   수정일: 2021-11-26 04:01:22 &lt;/Document-Metadata&gt;  [Sheet: 정리본] [Table Chunk 7/…</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -3892,26 +3892,26 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[0346542e0be2b2ab] 2024년도_(붙임 2) 2024 말용도 다각화 추진계획_본문 #12  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-23 09:05:49   수정일: 2024-06-01 17:42:54 &lt;/Documen
-[123f03df3479517e] 2022년도_[별첨1] KRA-ESG경영 진단모델(세부 진단기준)_최종 #43  ▸  &lt;Document-Metadata&gt;   제목: 《 KRA   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-04 14:33:57   수정일: 2023-05-27 10:21:04 &lt;/Docume
-[156fec294ba67ae4] 2024년도_★ (본문) 2024년 부경 경주마 보건복지 고도화 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2024-05-04 14:09:56 &lt;/Document-M
-[210e0e2db641965a] 2020년도_[붙임 1] 2020년 재활승마 활성화 지원 시범사업 계획(안_요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 말산업육성본부   작성자: KRA   마지막 수정자: KRA   작성일: 2017-05-24 17:59:41   수정일: 2020-08-07 15:31:04 &lt;/Docu
-[2212a005847a8f98] 2023년도_2023년 힐링승마 지원사업 추진 계획(안)_220308_2 #43  ▸  &lt;Document-Metadata&gt;   제목: 목 적   작성자: KRA   설명: |Fasoo_Trace_ID:eyJub2RlMSI6eyJkc2QiOiIwMTAwMDAwMDAwMDAxODMwIiwibG9nVGltZ
-[27dcbb61e82d6f82] 2024년도_과제 및 사업별 담당부서 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-08 02:27:01   수정일: 2024-06-13 05:02:20 &lt;/Document-Metadata&gt;
-[2a67e1073fe83029] 2022년도_2022 힐링승마 지원사업 운영 결과보고_221222 #25  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-08-06 09:18:55   수정일: 2022-12-22 18:09:26 &lt;/Document-Metadata&gt;
-[2d94f6c769030bda] 2020년도_경주마 통합 건강관리시스템 추진계획(안) #19  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2020-05-27 10:31:20 &lt;/Document-M
-[33882770624ec69f] 2022년도_「말의 인도적인 처리 가이드라인」수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2022-12-21 14:48:38 &lt;/Document-M
-[345beb807d95ba70] 2020년도_★(결재) 2020 사회공익힐링 승마 사업 기본 운영 계획 #5  ▸  &lt;Document-Metadata&gt;   제목: 2019 전국민 승마체험 사업 기본계획   작성자: user   마지막 수정자: KRA   작성일: 2019-02-15 13:56:48   수정일: 2020-02-26
-[386c3d238d9e12b0] 2021년도_(요약) 2021 사회공익 힐링승마 사업 결과보고 #4  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-23 17:48:23 &lt;/Document-M
-[3b4dc85349de4eae] 2023년도_(요약) 말등록부 연간 업무 추진계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-21 11:12:57 &lt;/Document-M
-[3fe2d89ca01994f0] 2023년도_[붙임1] 해외종축개발운영위원회규정 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: 2170058   작성일: 2014-08-15 11:42:18   수정일: 2024-05-26 10:50:28 &lt;/Docume
-[40122ffcb05effea] 2020년도_★(요약) 2020 사회공익힐링 승마 사업 기본 운영 계획 #10  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-04 13:13:33   수정일: 2020-02-26 16:19:50 &lt;/Document-Metadata&gt;
-[4c2beab48a4fa8ba] 2020년도_200304 (보고)2020년도 재활힐링승마 사업 전략적 홍보방안ver.5 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-05 15:19:27 &lt;/Document-M
-[4cb0ece55fc920e7] 2023년도_(요약) 2023년 말복지센터 업무 추진계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 2022   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-18 10:11:25   수정일: 2023-02-09 09:59:44 &lt;/Documen
-[4f2b02c85a84bf0f] 2024년도_2. 2024년 경주마 토탈 케어시스템 운영 계획(안) 1부 #23  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-02-04 09:56:05 &lt;/Document-Met
-[4f5b39b0938daff2] 2024년도_(붙임 1) 말용도 다각화 추진계획_요약 #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-06-01 17:40:16 &lt;/Document-M
-[54275dff6b495fb6] 2024년도_1. 2024년 경주마 토탈 케어시스템 운영 계획(안) 1부(요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 2022   작성자: KRA   마지막 수정자: KRA   작성일: 2022-04-17 09:56:03   수정일: 2024-02-03 17:32:13 &lt;/Documen
-[551eb387c7145222] 2024년도_[붙임1] 해외종축개발운영위원회규정 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: 2170058   작성일: 2014-08-15 11:42:18   수정일: 2024-05-26 10:50:28 &lt;/Docume
+          <t>1. 2024년도_(붙임 2) 2024 말용도 다각화 추진계획_본문 #12  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-23 09:05:49   수정일: 2024-06-01 17:42:54 &lt;/Document-Metadata&gt;  (단, 사업담당자의 재량으로 지…
+2. 2022년도_[별첨1] KRA-ESG경영 진단모델(세부 진단기준)_최종 #43  ▸  &lt;Document-Metadata&gt;   제목: 《 KRA   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-04 14:33:57   수정일: 2023-05-27 10:21:04 &lt;/Document-Metadata&gt;  &lt;table border='1…
+3. 2024년도_★ (본문) 2024년 부경 경주마 보건복지 고도화 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2024-05-04 14:09:56 &lt;/Document-Metadata&gt;  (치료) 복지중심 의료서비스 지원 강…
+4. 2020년도_[붙임 1] 2020년 재활승마 활성화 지원 시범사업 계획(안_요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 말산업육성본부   작성자: KRA   마지막 수정자: KRA   작성일: 2017-05-24 17:59:41   수정일: 2020-08-07 15:31:04 &lt;/Document-Metadata&gt;  [Image:temp/im…
+5. 2023년도_2023년 힐링승마 지원사업 추진 계획(안)_220308_2 #43  ▸  &lt;Document-Metadata&gt;   제목: 목 적   작성자: KRA   설명: |Fasoo_Trace_ID:eyJub2RlMSI6eyJkc2QiOiIwMTAwMDAwMDAwMDAxODMwIiwibG9nVGltZSI6IjIwMjItMDEtMjJUMDE6MzM6MjB…
+6. 2024년도_과제 및 사업별 담당부서 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-08 02:27:01   수정일: 2024-06-13 05:02:20 &lt;/Document-Metadata&gt;  [Sheet: 과제 및 사업별 담당] [Table …
+7. 2022년도_2022 힐링승마 지원사업 운영 결과보고_221222 #25  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-08-06 09:18:55   수정일: 2022-12-22 18:09:26 &lt;/Document-Metadata&gt;  &lt; 하반기 현장점검 결과 및 의견 &gt;  &lt;table…
+8. 2020년도_경주마 통합 건강관리시스템 추진계획(안) #19  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2020-05-27 10:31:20 &lt;/Document-Metadata&gt;  === Extracted Images…
+9. 2022년도_「말의 인도적인 처리 가이드라인」수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2022-12-21 14:48:38 &lt;/Document-Metadata&gt;  「말의 인도적인 처리 가이드라인」수립…
+10. 2020년도_★(결재) 2020 사회공익힐링 승마 사업 기본 운영 계획 #5  ▸  &lt;Document-Metadata&gt;   제목: 2019 전국민 승마체험 사업 기본계획   작성자: user   마지막 수정자: KRA   작성일: 2019-02-15 13:56:48   수정일: 2020-02-26 18:10:51 &lt;/Document-Metadata&gt; …
+11. 2021년도_(요약) 2021 사회공익 힐링승마 사업 결과보고 #4  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-23 17:48:23 &lt;/Document-Metadata&gt;  * 스트레스 감소 인원 대상 강습 전…
+12. 2023년도_(요약) 말등록부 연간 업무 추진계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-21 11:12:57 &lt;/Document-Metadata&gt;  3. 소요예산 : 438백만원 (마사…
+13. 2023년도_[붙임1] 해외종축개발운영위원회규정 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: 2170058   작성일: 2014-08-15 11:42:18   수정일: 2024-05-26 10:50:28 &lt;/Document-Metadata&gt;  &lt;table border='1…
+14. 2020년도_★(요약) 2020 사회공익힐링 승마 사업 기본 운영 계획 #10  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-04 13:13:33   수정일: 2020-02-26 16:19:50 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+15. 2020년도_200304 (보고)2020년도 재활힐링승마 사업 전략적 홍보방안ver.5 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-05 15:19:27 &lt;/Document-Metadata&gt;  ○ 찾아가는 사회공익힐링승마 (상반기…
+16. 2023년도_(요약) 2023년 말복지센터 업무 추진계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 2022   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-18 10:11:25   수정일: 2023-02-09 09:59:44 &lt;/Document-Metadata&gt;  * `23년 마주출연 기금(10…
+17. 2024년도_2. 2024년 경주마 토탈 케어시스템 운영 계획(안) 1부 #23  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-02-04 09:56:05 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr…
+18. 2024년도_(붙임 1) 말용도 다각화 추진계획_요약 #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-06-01 17:40:16 &lt;/Document-Metadata&gt;  ㅇ 지원대상 : 국내 말 등록기관*에…
+19. 2024년도_1. 2024년 경주마 토탈 케어시스템 운영 계획(안) 1부(요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 2022   작성자: KRA   마지막 수정자: KRA   작성일: 2022-04-17 09:56:03   수정일: 2024-02-03 17:32:13 &lt;/Document-Metadata&gt;  2024년 경주마 토탈 케어시스…
+20. 2024년도_[붙임1] 해외종축개발운영위원회규정 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: 2170058   작성일: 2014-08-15 11:42:18   수정일: 2024-05-26 10:50:28 &lt;/Document-Metadata&gt;  &lt;table border='1…
 ... +47 more</t>
         </is>
       </c>
@@ -4019,18 +4019,18 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[1c2e14b3e46641c4] 2023년도_(붙임1) 말산업 일학습병행제 도입 및 활성화 추진경과 #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-09-08 16:25:03 &lt;/Document-M
-[33ad8cb9e391ffb3] 2020년도_(붙임#1) 인재개발 기본계획(안) 요약 #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-27 16:38:24 &lt;/Documen
-[34ee099eaee5f3ae] 2022년도_(본문) 경주마관계자 임시조치 개선계획(안) #34  ▸  &lt;Document-Metadata&gt;   제목: 2022년 교육훈련 기본계획   작성자: KRA   마지막 수정자: KRA   작성일: 2022-03-04 14:47:46   수정일: 2022-11-11 16:14:3
-[3c78d27b62aca0f0] 2022년도_(붙임1) 말산업 일학습병행제 도입 및 활성화 추진경과 #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-09-08 16:25:03 &lt;/Document-M
-[5cf871e3bcad9e3b] 2025년도_(붙임3) 2025년 한국마사회 수입 및 지출계획서 #12  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2024-12-19 17:06:39 &lt;/Documen
-[6348ecdf3dc5e21e] 2024년도_[요약] 24년 데이터기반행정 활성화 추진계획_240504 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-05-04 09:27:45 &lt;/Document-M
-[7397f4cf3cd4bcb4] 2022년도_(붙임4) 2023년 경마분야 지원 R&amp;D 추진계획(최종) #14  ▸  &lt;Document-Metadata&gt;   제목: 시험시행 종합계획   작성자: KRA   마지막 수정자: KRA   작성일: 2012-07-27 11:07:39   수정일: 2023-06-17 13:39:57 &lt;/Do
-[750220b64c1d0833] 2022년도_(경마본부) 2022년 핵심과제 추진실적 #4  ▸  &lt;Document-Metadata&gt;   제목: 감사원 지적사항 조치실적   마지막 수정자: KRA   작성일: 2007-12-13 21:52:10   수정일: 2022-12-20 10:42:23 &lt;/Document-
-[790f2015dc65b6e1] 2020년도_(붙임#2) 2020년 인재개발 기본계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 인 사 노 무 처   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-02 10:20:11   수정일: 2020-02-27 16:52:55 &lt;/Do
-[811aee113d51f0a0] 2023년도_(붙임4) 2023년 경마분야 지원 R&amp;D 추진계획(최종) #14  ▸  &lt;Document-Metadata&gt;   제목: 시험시행 종합계획   작성자: KRA   마지막 수정자: KRA   작성일: 2012-07-27 11:07:39   수정일: 2023-06-17 13:39:57 &lt;/Do
-[c13ca063e2675d57] 2022년도_1. 경마안정성 강화 대책 수립 계획(안) #5  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-18 19:10:02   수정일: 2023-02-04 17:46:47 &lt;/Documen
-[d91964b859494daf] 2021년도_(붙임3)_2021년도 수입 및 지출 계획서 #14  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2020-12-18 18:13:07 &lt;/Documen</t>
+          <t>1. 2023년도_(붙임1) 말산업 일학습병행제 도입 및 활성화 추진경과 #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-09-08 16:25:03 &lt;/Document-Metadata&gt;  * 산업형(100% NCS 적용) 채…
+2. 2020년도_(붙임#1) 인재개발 기본계획(안) 요약 #0  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-27 16:38:24 &lt;/Document-Metadata&gt;  2020년 인재개발 기본계획(안…
+3. 2022년도_(본문) 경주마관계자 임시조치 개선계획(안) #34  ▸  &lt;Document-Metadata&gt;   제목: 2022년 교육훈련 기본계획   작성자: KRA   마지막 수정자: KRA   작성일: 2022-03-04 14:47:46   수정일: 2022-11-11 16:14:31 &lt;/Document-Metadata&gt;  Ⅶ. 협조사…
+4. 2022년도_(붙임1) 말산업 일학습병행제 도입 및 활성화 추진경과 #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-09-08 16:25:03 &lt;/Document-Metadata&gt;  * 산업형(100% NCS 적용) 채…
+5. 2025년도_(붙임3) 2025년 한국마사회 수입 및 지출계획서 #12  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2024-12-19 17:06:39 &lt;/Document-Metadata&gt;  훈), 예산담당사원(강현석)  …
+6. 2024년도_[요약] 24년 데이터기반행정 활성화 추진계획_240504 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-05-04 09:27:45 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+7. 2022년도_(붙임4) 2023년 경마분야 지원 R&amp;D 추진계획(최종) #14  ▸  &lt;Document-Metadata&gt;   제목: 시험시행 종합계획   작성자: KRA   마지막 수정자: KRA   작성일: 2012-07-27 11:07:39   수정일: 2023-06-17 13:39:57 &lt;/Document-Metadata&gt;  선정 가능성 체크리스트…
+8. 2022년도_(경마본부) 2022년 핵심과제 추진실적 #4  ▸  &lt;Document-Metadata&gt;   제목: 감사원 지적사항 조치실적   마지막 수정자: KRA   작성일: 2007-12-13 21:52:10   수정일: 2022-12-20 10:42:23 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; …
+9. 2020년도_(붙임#2) 2020년 인재개발 기본계획(안) #8  ▸  &lt;Document-Metadata&gt;   제목: 인 사 노 무 처   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-02 10:20:11   수정일: 2020-02-27 16:52:55 &lt;/Document-Metadata&gt;  &lt;table borde…
+10. 2023년도_(붙임4) 2023년 경마분야 지원 R&amp;D 추진계획(최종) #14  ▸  &lt;Document-Metadata&gt;   제목: 시험시행 종합계획   작성자: KRA   마지막 수정자: KRA   작성일: 2012-07-27 11:07:39   수정일: 2023-06-17 13:39:57 &lt;/Document-Metadata&gt;  선정 가능성 체크리스트…
+11. 2022년도_1. 경마안정성 강화 대책 수립 계획(안) #5  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-18 19:10:02   수정일: 2023-02-04 17:46:47 &lt;/Document-Metadata&gt;  (대고객 사과) 1.15(일) …
+12. 2021년도_(붙임3)_2021년도 수입 및 지출 계획서 #14  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2020-12-18 18:13:07 &lt;/Document-Metadata&gt;  재원), 예산담당대리(권오경) …</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -4082,26 +4082,26 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[0346542e0be2b2ab] 2024년도_(붙임 2) 2024 말용도 다각화 추진계획_본문 #12  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-23 09:05:49   수정일: 2024-06-01 17:42:54 &lt;/Documen
-[0370e8a4dce03ce3] 2020년도_경마실황 무선중계시스템 도입 계획(안) #9  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-20 12:54:03   수정일: 2020-08-08 11:33:53 &lt;/Document-Metadata&gt;
-[08712ddb117bedbb] 2023년도_2023 온라인 방송 추진 계획(안)_최종 #12  ▸  &lt;Document-Metadata&gt;   제목: 미래비전의 초석   작성자: KRA   마지막 수정자: KRA   작성일: 2022-05-28 14:52:15   수정일: 2023-07-23 09:58:23 &lt;/Doc
-[123f03df3479517e] 2022년도_[별첨1] KRA-ESG경영 진단모델(세부 진단기준)_최종 #43  ▸  &lt;Document-Metadata&gt;   제목: 《 KRA   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-04 14:33:57   수정일: 2023-05-27 10:21:04 &lt;/Docume
-[133dd2fda4f7c41d] 2024년도_(붙임 1) 제1회 국산마 품평회 개최계획 #18  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-15 17:31:04   수정일: 2024-06-19 17:49:01 &lt;/Documen
-[156fec294ba67ae4] 2024년도_★ (본문) 2024년 부경 경주마 보건복지 고도화 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2024-05-04 14:09:56 &lt;/Document-M
-[17a6323f30b615ff] 2024년도_(요약) 보고서(2024년 부경본부 후반기 입장인원 증대계획) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2024-07-24 17:56:30 &lt;/Document-Metadat
-[1e7df0e389317f02] 2024년도_2024년 봄 야간경마 시즌 드라이브 스루 베팅존 운영계획(안) 240225 결재 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:54:36   수정일: 2024-02-25 16:31:26 &lt;/Document-M
-[24fa325d76c7cd8a] 2024년도_2024년 서울경마공원 발매사업 운영계획(안)_최종 #0  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2024-03-22 09:44:13 &lt;/Docume
-[2965f2e46bcfa371] 2024년도_(붙임1) 제주 경마방송 노후 동기 신호 발생기 교체 계획(안)_V2 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-18 09:43:45   수정일: 2024-05-12 16:07:00 &lt;/Document-M
-[2e907c84c2a15612] 2021년도_K-TOTE 클라우드 전환 구축 시행계획(요약)_최종 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-06-17 10:42:08 &lt;/Document-M
-[30e5c01f74f2a2b2] 2024년도_2024년 발매사업 운영계획(안)_ver3.0 #16  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2024-03-03 16:48:21 &lt;/Docume
-[329af5c7de78350a] 2024년도_(붙임) 2024년 인권경영 기본계획(안)_240414★ #2  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2024-04-16 16:56:55 &lt;/Documen
-[3899cc22b412106f] 2022년도_(친환경탄소중립) 2022 보고서 작성_환경_5차 워크숍_컨설팅_최종 #40  ▸  &lt;Document-Metadata&gt;   제목: 1. 전략기획 및 사회적책임   마지막 수정자: KRA   작성일: 2015-01-15 14:27:57   수정일: 2023-02-19 14:55:17 &lt;/Documen
-[38bd220368aba4ab] 2023년도_[붙임 1] (요약) 말산업 R&amp;D 중장기 로드맵 구축 연구 #10  ▸  &lt;Document-Metadata&gt;   제목: 사업개요   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-19 15:06:14   수정일: 2024-03-03 16:48:29 &lt;/Documen
-[3d8c8292183997c8] 2023년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-M
-[3e1e3c7c7c6dbc28] 2024년도_[붙임2] 개정 「내부통제규정」전문 #10  ▸  &lt;Document-Metadata&gt;   제목: 제1장  총칙                                      작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-28 17:38:1
-[3f4afc51b550193f] 2023년도_2. [본문] 2023년 영향평가 시행 계획(안) #15  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2023-05-18 09:24:05 &lt;/Document-Met
-[3fb6428d743036ee] 2022년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-M
-[419a0013fb52efe2] 2024년도_(요약)'24년 안전보건경영시스템 경영자 검토보고 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-28 16:47:06   수정일: 2024-12-27 09:58:43 &lt;/Document-Metadata&gt;
+          <t>1. 2024년도_(붙임 2) 2024 말용도 다각화 추진계획_본문 #12  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-23 09:05:49   수정일: 2024-06-01 17:42:54 &lt;/Document-Metadata&gt;  (단, 사업담당자의 재량으로 지…
+2. 2020년도_경마실황 무선중계시스템 도입 계획(안) #9  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-20 12:54:03   수정일: 2020-08-08 11:33:53 &lt;/Document-Metadata&gt;  나. 계약 방법 : 견적 최저가       LTE …
+3. 2023년도_2023 온라인 방송 추진 계획(안)_최종 #12  ▸  &lt;Document-Metadata&gt;   제목: 미래비전의 초석   작성자: KRA   마지막 수정자: KRA   작성일: 2022-05-28 14:52:15   수정일: 2023-07-23 09:58:23 &lt;/Document-Metadata&gt;  ❍ 내용 : 온라인 발매…
+4. 2022년도_[별첨1] KRA-ESG경영 진단모델(세부 진단기준)_최종 #43  ▸  &lt;Document-Metadata&gt;   제목: 《 KRA   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-04 14:33:57   수정일: 2023-05-27 10:21:04 &lt;/Document-Metadata&gt;  &lt;table border='1…
+5. 2024년도_(붙임 1) 제1회 국산마 품평회 개최계획 #18  ▸  &lt;Document-Metadata&gt;   제목: 2024   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-15 17:31:04   수정일: 2024-06-19 17:49:01 &lt;/Document-Metadata&gt;  소요예산 : 97,200천원  …
+6. 2024년도_★ (본문) 2024년 부경 경주마 보건복지 고도화 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2017-09-16 17:23:25   수정일: 2024-05-04 14:09:56 &lt;/Document-Metadata&gt;  (치료) 복지중심 의료서비스 지원 강…
+7. 2024년도_(요약) 보고서(2024년 부경본부 후반기 입장인원 증대계획) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2024-07-24 17:56:30 &lt;/Document-Metadata&gt;  (요약) (부경본부) 2024년 후반기 입장인원…
+8. 2024년도_2024년 봄 야간경마 시즌 드라이브 스루 베팅존 운영계획(안) 240225 결재 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:54:36   수정일: 2024-02-25 16:31:26 &lt;/Document-Metadata&gt;  , 매출액(101백만원)       …
+9. 2024년도_2024년 서울경마공원 발매사업 운영계획(안)_최종 #0  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2024-03-22 09:44:13 &lt;/Document-Metadata&gt;  &lt;table border='1…
+10. 2024년도_(붙임1) 제주 경마방송 노후 동기 신호 발생기 교체 계획(안)_V2 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-18 09:43:45   수정일: 2024-05-12 16:07:00 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+11. 2021년도_K-TOTE 클라우드 전환 구축 시행계획(요약)_최종 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-06-17 10:42:08 &lt;/Document-Metadata&gt;  □ 추진기간 : 2021. 6월 ∼ …
+12. 2024년도_2024년 발매사업 운영계획(안)_ver3.0 #16  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2024-03-03 16:48:21 &lt;/Document-Metadata&gt;  &lt;table border='1…
+13. 2024년도_(붙임) 2024년 인권경영 기본계획(안)_240414★ #2  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2024-04-16 16:56:55 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+14. 2022년도_(친환경탄소중립) 2022 보고서 작성_환경_5차 워크숍_컨설팅_최종 #40  ▸  &lt;Document-Metadata&gt;   제목: 1. 전략기획 및 사회적책임   마지막 수정자: KRA   작성일: 2015-01-15 14:27:57   수정일: 2023-02-19 14:55:17 &lt;/Document-Metadata&gt;  [Image:temp/image…
+15. 2023년도_[붙임 1] (요약) 말산업 R&amp;D 중장기 로드맵 구축 연구 #10  ▸  &lt;Document-Metadata&gt;   제목: 사업개요   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-19 15:06:14   수정일: 2024-03-03 16:48:29 &lt;/Document-Metadata&gt;  === Extracted Ima…
+16. 2023년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-Metadata&gt;  전환에 대비한 시공간 제약 없는 원격…
+17. 2024년도_[붙임2] 개정 「내부통제규정」전문 #10  ▸  &lt;Document-Metadata&gt;   제목: 제1장  총칙                                      작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-28 17:38:15   수정일: 2024-12-14 09:38:18 &lt;…
+18. 2023년도_2. [본문] 2023년 영향평가 시행 계획(안) #15  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2023-05-18 09:24:05 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr…
+19. 2022년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-Metadata&gt;  전환에 대비한 시공간 제약 없는 원격…
+20. 2024년도_(요약)'24년 안전보건경영시스템 경영자 검토보고 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-28 16:47:06   수정일: 2024-12-27 09:58:43 &lt;/Document-Metadata&gt;  5. 향후계획 : 차년도 산업안전보건 계획 수립 시…
 ... +67 more</t>
         </is>
       </c>
@@ -4229,28 +4229,28 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[030292b5e5db1492] 2023년도_(요약본) 2023년 기록관리 기본계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-03-30 09:55:50 &lt;/Document-M
-[06b38c6a346a2385] 2023년도_2023년 바로마켓 운영 계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2011-01-14 09:36:36   수정일: 2023-02-05 17:18:03 &lt;/Document-M
-[06ea8eb0c6498c61] 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-M
-[0f9e1947b0221b27] 2023년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-M
-[1002c0855b631621] 2022년도_한국마사회 ESG경영부 2022년 인권경영 이행실적 보고서 견적서 #1  ▸  &lt;Document-Metadata&gt;   작성자: Administrator   마지막 수정자: 이주훈   작성일: 2012-01-19 08:40:24   수정일: 2023-06-18 09:36:47 &lt;/Document
-[10f09627fe81dec0] 2024년도_2024 마권 용지 및 구매표 구매 계획 요약 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-22 11:16:41 &lt;/Document-M
-[1288cb8b3a80b7a4] 2025년도_[요약] 2025년 학교체육 승마 지원사업 운영계획(안) 241201 #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-12-01 14:34:19 &lt;/Document-M
-[19fa870b8e483f1c] 2024년도_512.기부금관리규정(전문) #31  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
+          <t>1. 2023년도_(요약본) 2023년 기록관리 기본계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-03-30 09:55:50 &lt;/Document-Metadata&gt;  3. 2023년 기본계획 (안)   …
+2. 2023년도_2023년 바로마켓 운영 계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2011-01-14 09:36:36   수정일: 2023-02-05 17:18:03 &lt;/Document-Metadata&gt;  *바로마켓 사용료 산출산식 : 참여농…
+3. 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-Metadata&gt;  가와 사업성과평가 통합    ◦ (차…
+4. 2023년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+5. 2022년도_한국마사회 ESG경영부 2022년 인권경영 이행실적 보고서 견적서 #1  ▸  &lt;Document-Metadata&gt;   작성자: Administrator   마지막 수정자: 이주훈   작성일: 2012-01-19 08:40:24   수정일: 2023-06-18 09:36:47 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt;…
+6. 2024년도_2024 마권 용지 및 구매표 구매 계획 요약 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-22 11:16:41 &lt;/Document-Metadata&gt;  : 현 재고량(4,754 BOX)에 …
+7. 2025년도_[요약] 2025년 학교체육 승마 지원사업 운영계획(안) 241201 #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-12-01 14:34:19 &lt;/Document-Metadata&gt;  전학년 20명 이하의 학교    ❍ …
+8. 2024년도_512.기부금관리규정(전문) #31  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
     설명: 
-    마지막 수정자: KRA   작성일: 2006-03-14 14:40:25   수정일: 2024-12-05 18:
-[1a1522e81a560fbf] 2020년도_(본문)20년 말산업 컨설팅 추진계획(안) #32  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2015-02-08 08:46:52   수정일: 2020-03-25 11:26:26 &lt;/Document-Metadata&gt;
-[1c82399b98aebbba] 2024년도_(양식) 상반기 자본예산 집행실적 #21  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-05 10:21:26   수정일: 2024-06-13 06:23:29 &lt;/Document-Metadata&gt;
-[1d6b0fc02595dbd7] 2020년도_(요약) 2020 한국경마 대국민 인식조사 결과보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-01-28 13:35:00 &lt;/Document-M
-[2170040846621df2] 2020년도_붙임 2.  2020 박람회추진계획(안)(요약) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-27 10:42:10 &lt;/Document-M
-[21a9f52b725a25b7] 2021년도_20210327 2021년 바로마켓 운영 계획(안) 요약보고 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-03-27 17:30:56 &lt;/Document-M
-[23f259fe9f9c25d9] 2020년도_200828_언택트발매추진단 하반기 사업계획 및 예산 #4  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-21 12:13:34   수정일: 2020-08-28 13:15:23 &lt;/Document-M
-[2520e4f72ad580ae] 2022년도_(제23-11호) 인권경영 실행지침 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-04 09:10:19   수정일: 2023-04-23 10:51:13 &lt;/Do
-[257c21115efd0262] 2022년도_2022년도 기관경영평가 재무예산관리 지표 경영실적보고서(수정, 02.18) #96  ▸  &lt;Document-Metadata&gt;   제목: 1. 전략기획 및 사회적책임   마지막 수정자: KRA   작성일: 2015-01-15 14:27:57   수정일: 2023-02-18 17:30:08 &lt;/Documen
-[26804b9bb678ce82] 2020년도_('20.08.06) 공공기관 자회사 운영실태 평가 계획(비대면) #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-08-09 15:07:56 &lt;/Document-M
-[2a3a0e1ad3162f25] 2024년도_(붙임2) '24년 마권용지 및 구매표 구매계획(안)_최종 #24  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2011-03-04 12:47:46   수정일: 2024-02-22 11:20:58 &lt;/Document-M
-[2e907c84c2a15612] 2021년도_K-TOTE 클라우드 전환 구축 시행계획(요약)_최종 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-06-17 10:42:08 &lt;/Document-M
-[2ffc5467d8f17d86] 2020년도_(본문) 2020년 한국마사회 지식경영 운영계획(안)(200417) #19  ▸  &lt;Document-Metadata&gt;   제목: 2017년 지식경영 운영계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-13 15:38:51   수정일: 2020-04-17 10:22:3
+    마지막 수정자: KRA   작성일: 2006-03-14 14:40:25   수정일: 2024-12-05 18:46:10 &lt;/Document-Metadata&gt;  ※ …
+9. 2020년도_(본문)20년 말산업 컨설팅 추진계획(안) #32  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2015-02-08 08:46:52   수정일: 2020-03-25 11:26:26 &lt;/Document-Metadata&gt;  [Image:temp/images/hwp_BIN00…
+10. 2024년도_(양식) 상반기 자본예산 집행실적 #21  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-05 10:21:26   수정일: 2024-06-13 06:23:29 &lt;/Document-Metadata&gt;  [Sheet: Sheet1] [Table 3] | …
+11. 2020년도_(요약) 2020 한국경마 대국민 인식조사 결과보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-01-28 13:35:00 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+12. 2020년도_붙임 2.  2020 박람회추진계획(안)(요약) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-27 10:42:10 &lt;/Document-Metadata&gt;  □ (융‧복합형) 비즈니스 산업과 엔…
+13. 2021년도_20210327 2021년 바로마켓 운영 계획(안) 요약보고 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-03-27 17:30:56 &lt;/Document-Metadata&gt;  -‘20년도 정상개장(워킹스루) : …
+14. 2020년도_200828_언택트발매추진단 하반기 사업계획 및 예산 #4  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-21 12:13:34   수정일: 2020-08-28 13:15:23 &lt;/Document-Metadata&gt;  및 말산업 생태계 보존     (이용…
+15. 2022년도_(제23-11호) 인권경영 실행지침 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-04 09:10:19   수정일: 2023-04-23 10:51:13 &lt;/Document-Metadata&gt;  동과 아동노동도 허용하…
+16. 2022년도_2022년도 기관경영평가 재무예산관리 지표 경영실적보고서(수정, 02.18) #96  ▸  &lt;Document-Metadata&gt;   제목: 1. 전략기획 및 사회적책임   마지막 수정자: KRA   작성일: 2015-01-15 14:27:57   수정일: 2023-02-18 17:30:08 &lt;/Document-Metadata&gt;  [Image:temp/image…
+17. 2020년도_('20.08.06) 공공기관 자회사 운영실태 평가 계획(비대면) #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-08-09 15:07:56 &lt;/Document-Metadata&gt;  「고용부, 자회사 운영 실태평가 」지…
+18. 2024년도_(붙임2) '24년 마권용지 및 구매표 구매계획(안)_최종 #24  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: kra   마지막 수정자: KRA   작성일: 2011-03-04 12:47:46   수정일: 2024-02-22 11:20:58 &lt;/Document-Metadata&gt;  * 최종 단가는 경쟁입찰 낙찰단가를 …
+19. 2021년도_K-TOTE 클라우드 전환 구축 시행계획(요약)_최종 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-06-17 10:42:08 &lt;/Document-Metadata&gt;  □ 추진기간 : 2021. 6월 ∼ …
+20. 2020년도_(본문) 2020년 한국마사회 지식경영 운영계획(안)(200417) #19  ▸  &lt;Document-Metadata&gt;   제목: 2017년 지식경영 운영계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-13 15:38:51   수정일: 2020-04-17 10:22:34 &lt;/Document-Metadata&gt;  부서 심사 …
 ... +113 more</t>
         </is>
       </c>
@@ -4424,17 +4424,17 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[08dbb848822964aa] 2024년도_(요약)2024년 승용마 번식 지원사업 추진계획(안) #0  ▸  &lt;Document-Metadata&gt;   제목: CEO지시사항 추진과제 입력 매뉴얼   작성자: kra   마지막 수정자: KRA   작성일: 2014-03-29 09:25:36   수정일: 2024-04-05 08:
-[2b77cb92e3b2e52e] 2020년도_붙임3. 2020년 총 교배횟수(모든교배내역) #144  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:38:42 &lt;/Document-Metadata&gt;
-[43b8261fe9a4b3ca] 2020년도_@ (결재상신) 2020년 경주마 생산 및 교배지원 결과보고 @ #19  ▸  &lt;Document-Metadata&gt;   제목: 2002. 내륙 민간목장 생산 및 교배지원 결과   작성자: 한국마사회 원당목장팀 대리 임진호   키워드: 
+          <t>1. 2024년도_(요약)2024년 승용마 번식 지원사업 추진계획(안) #0  ▸  &lt;Document-Metadata&gt;   제목: CEO지시사항 추진과제 입력 매뉴얼   작성자: kra   마지막 수정자: KRA   작성일: 2014-03-29 09:25:36   수정일: 2024-04-05 08:50:21 &lt;/Document-Metadata&gt;  20…
+2. 2020년도_붙임3. 2020년 총 교배횟수(모든교배내역) #144  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:38:42 &lt;/Document-Metadata&gt;  [Sheet: 2020 총 교배횟수] [Table …
+3. 2020년도_@ (결재상신) 2020년 경주마 생산 및 교배지원 결과보고 @ #19  ▸  &lt;Document-Metadata&gt;   제목: 2002. 내륙 민간목장 생산 및 교배지원 결과   작성자: 한국마사회 원당목장팀 대리 임진호   키워드: 
     설명: 
-    마지막 수정자: KRA
-[481cdea45e2aa69d] 2020년도_붙임1. 2020년 경주마 생산실적 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:32:35 &lt;/Document-Metadata&gt;
-[57ae80a2b693d18f] 2020년도_붙임4. 2020년 유상교배 수익내역 #6  ▸  &lt;Document-Metadata&gt;   작성자: user   마지막 수정자: KRA   작성일: 2013-10-13 05:56:53   수정일: 2020-12-11 01:28:30 &lt;/Document-Metadata
-[6cdb3f17c1eafe48] 2020년도_붙임2. 2020년 총 교배실적(두수) #111  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:36:12 &lt;/Document-Metadata&gt;
-[72b1245e55ab96fc] 2021년도_경주마 교배 및 번식분야 복지 가이드라인(안) #17  ▸  &lt;Document-Metadata&gt;   제목: 한국마사회 교배 및 번식 말 복지 가이드라인 초안    작성자: User2007   마지막 수정자: KRA   작성일: 2021-08-07 21:34:58   수정일:
-[bbe40d855e6cc165] 2021년도_경주마 교배 및 번식분야 복지 가이드라인 수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-02 15:44:31 &lt;/Document-M
-[e39b4656a5219700] 2020년도_@ (요약) 2020년 경주마 생산 및 교배지원 결과보고 @ #3  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-12-17 11:13:23 &lt;/Document-Metadat</t>
+    마지막 수정자: KRA   작성일: 2005-08-25 10:09:53   수정…
+4. 2020년도_붙임1. 2020년 경주마 생산실적 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:32:35 &lt;/Document-Metadata&gt;  [Sheet: 2020년 생산내역 (수정)] [Ta…
+5. 2020년도_붙임4. 2020년 유상교배 수익내역 #6  ▸  &lt;Document-Metadata&gt;   작성자: user   마지막 수정자: KRA   작성일: 2013-10-13 05:56:53   수정일: 2020-12-11 01:28:30 &lt;/Document-Metadata&gt;  [Sheet: 작업용] [Table Chunk 7…
+6. 2020년도_붙임2. 2020년 총 교배실적(두수) #111  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-05 06:52:33   수정일: 2020-12-11 01:36:12 &lt;/Document-Metadata&gt;  [Sheet: 2020년 총 교배두수_최종교배기준]…
+7. 2021년도_경주마 교배 및 번식분야 복지 가이드라인(안) #17  ▸  &lt;Document-Metadata&gt;   제목: 한국마사회 교배 및 번식 말 복지 가이드라인 초안    작성자: User2007   마지막 수정자: KRA   작성일: 2021-08-07 21:34:58   수정일: 2021-12-02 11:22:35 &lt;/Document…
+8. 2021년도_경주마 교배 및 번식분야 복지 가이드라인 수립 결과 보고 #0  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-02 15:44:31 &lt;/Document-Metadata&gt;  경주마 교배 및 번식분야 복지 가이드…
+9. 2020년도_@ (요약) 2020년 경주마 생산 및 교배지원 결과보고 @ #3  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-12-17 11:13:23 &lt;/Document-Metadata&gt;  두, 민간 1,485두)      ○ 전체 대비…</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -4483,19 +4483,19 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[0f9e1947b0221b27] 2023년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-M
-[19fe4e04b9ae46af] 2023년도_붙임1.2024년 업무용 정보화기기 도입 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-05-26 17:28:25 &lt;/Document-Met
-[3d8c8292183997c8] 2023년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-M
-[3fb6428d743036ee] 2022년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-M
-[53036042c659a508] 2024년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-M
-[5b4cfb9e5eb0817f] 2024년도_붙임1.2024년 업무용 정보화기기 도입 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-05-26 17:28:25 &lt;/Document-Met
-[7d016a8eb300196a] 2024년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;
-[8c8f02475898d6e9] 2024년도_(요약)스마트 사무환경 고도화 추진 계획 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-21 11:12:09 &lt;/Document-M
-[993ad9a5e29994fc] 2023년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Documen
-[9d226cce773a4434] 2022년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Documen
-[a869fa35476990c2] 2023년도_서울경마공원 콜센터 설비 이중화 및 망분리 계획(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-09 11:14:17   수정일: 2024-04-06 17:02:38 &lt;/Document-Metadata&gt;
-[afd0f60cc9c978c0] 2022년도_붙임 1. 스마트 사무환경 구축 및 망분리 개선 견적서(총괄) #27  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-02 04:07:54   수정일: 2023-08-17 03:33:36 &lt;/Document-Metadata&gt;
-[e4f72caaf5619284] 2023년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2023년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+2. 2023년도_붙임1.2024년 업무용 정보화기기 도입 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-05-26 17:28:25 &lt;/Document-Metadata&gt;  [Image:temp/images/hwp…
+3. 2023년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-Metadata&gt;  전환에 대비한 시공간 제약 없는 원격…
+4. 2022년도_스마트 사무환경 구축(요약보고) #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-08-18 09:24:44 &lt;/Document-Metadata&gt;  전환에 대비한 시공간 제약 없는 원격…
+5. 2024년도_(요약)2024년 업무용 정보화기기 도입 계획 #1  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-05-26 17:28:55 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+6. 2024년도_붙임1.2024년 업무용 정보화기기 도입 계획(안) #0  ▸  &lt;Document-Metadata&gt;   작성자: (주)한글과컴퓨터   마지막 수정자: KRA   작성일: 2004-11-09 15:23:46   수정일: 2024-05-26 17:28:25 &lt;/Document-Metadata&gt;  [Image:temp/images/hwp…
+7. 2024년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;  [Sheet: 15년도 이하 소형복합기] [Tabl…
+8. 2024년도_(요약)스마트 사무환경 고도화 추진 계획 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-21 11:12:09 &lt;/Document-Metadata&gt;  최 운영부서 근무자 기준 약 450대…
+9. 2023년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Document-Metadata&gt;  [Image:temp/image…
+10. 2022년도_스마트 사무환경 구축 및 망분리 개선 추진계획(안) V1.0 #0  ▸  &lt;Document-Metadata&gt;   제목: 2023   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-08-18 09:26:47 &lt;/Document-Metadata&gt;  [Image:temp/image…
+11. 2023년도_서울경마공원 콜센터 설비 이중화 및 망분리 계획(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-09 11:14:17   수정일: 2024-04-06 17:02:38 &lt;/Document-Metadata&gt;  □ 예산과목: 노후통신시스템교체(1431040-24…
+12. 2022년도_붙임 1. 스마트 사무환경 구축 및 망분리 개선 견적서(총괄) #27  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-02 04:07:54   수정일: 2023-08-17 03:33:36 &lt;/Document-Metadata&gt;  [Sheet: 3.2 SSD] [Image:temp…
+13. 2023년도_붙임3.2024년도 교체대상 정보화기기 #13  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-05-26 04:02:11   수정일: 2024-05-26 04:49:07 &lt;/Document-Metadata&gt;  [Sheet: 15년도 이하 소형복합기] [Tabl…</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -4548,28 +4548,28 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[012dcbe84f52c595] 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Me
-[05dbe5ea6c8d03fe] 2024년도_(붙임3) 2024년 제주방송 프로그램 연간 제작계획 #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-02-02 04:18:57   수정일: 2024-01-26 05:46:09 &lt;/Document-Metadata&gt;
-[0787b40b4734cb4b] 2023년도_[붙임2] (본문) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #9  ▸  &lt;Document-Metadata&gt;   제목: 2019   작성자: KRA   마지막 수정자: KRA   작성일: 2019-07-24 15:06:06   수정일: 2024-05-25 09:18:53 &lt;/Documen
-[110f8ff7eb5dbdc1] 2022년도_첨부1_2022년 한국 대상경주 레이스 레이팅 총괄(연말최종) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-12-28 05:32:05   수정일: 2022-12-16 01:40:34 &lt;/Document-Metadata&gt;
-[134ceaf0ae1ba751] 2023년도_(요약) 23년 국제경주(코리아컵 코리아스프린트) 시행계획 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-04-28 10:50:47 &lt;/Document-M
-[22bf2d7e00a0f6d9] 2024년도_2024년 시리즈 경주 시행 결과보고 #25  ▸  &lt;Document-Metadata&gt;   제목: 대상경주 시리즈 선발체계 홍보   작성자: KRA   마지막 수정자: KRA   작성일: 2024-12-12 09:56:21   수정일: 2024-12-13 18:21:
-[2df376eb9253a430] 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Me
-[33640ab36a7a2b8c] 2024년도_2024년 제 2차 KPC 개최 심의 안건 #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-18 12:53:46 &lt;/Document-Metadata&gt;
-[517703ddbb49e0f6] 2024년도_붙임  (요약)야간경마 행사 추진계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-11 16:38:58 &lt;/Document-M
-[5d259d9a09f37c29] 2024년도_[붙임2] (본문) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #9  ▸  &lt;Document-Metadata&gt;   제목: 2019   작성자: KRA   마지막 수정자: KRA   작성일: 2019-07-24 15:06:06   수정일: 2024-05-25 09:18:53 &lt;/Documen
-[606afb85836eff9c] 2024년도_붙임2) (경주분류위원회)부의안건 #17  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-28 09:41:41 &lt;/Document-Metadata&gt;
-[6f3bfd6f2d2b9b04] 2022년도_(211230)2022_제주경마계획_책자원고(최종수정) #141  ▸  &lt;Document-Metadata&gt;   제목: Ⅱ. 경마 시행 개요   키워드: 
+          <t>1. 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…
+2. 2024년도_(붙임3) 2024년 제주방송 프로그램 연간 제작계획 #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-02-02 04:18:57   수정일: 2024-01-26 05:46:09 &lt;/Document-Metadata&gt;  [Sheet: Sheet1] [Table Chunk…
+3. 2023년도_[붙임2] (본문) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #9  ▸  &lt;Document-Metadata&gt;   제목: 2019   작성자: KRA   마지막 수정자: KRA   작성일: 2019-07-24 15:06:06   수정일: 2024-05-25 09:18:53 &lt;/Document-Metadata&gt;  === Extracted Ima…
+4. 2022년도_첨부1_2022년 한국 대상경주 레이스 레이팅 총괄(연말최종) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2017-12-28 05:32:05   수정일: 2022-12-16 01:40:34 &lt;/Document-Metadata&gt;  [Sheet: Sheet1] [Table Chunk…
+5. 2023년도_(요약) 23년 국제경주(코리아컵 코리아스프린트) 시행계획 #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2023-04-28 10:50:47 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+6. 2024년도_2024년 시리즈 경주 시행 결과보고 #25  ▸  &lt;Document-Metadata&gt;   제목: 대상경주 시리즈 선발체계 홍보   작성자: KRA   마지막 수정자: KRA   작성일: 2024-12-12 09:56:21   수정일: 2024-12-13 18:21:21 &lt;/Document-Metadata&gt;  === E…
+7. 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…
+8. 2024년도_2024년 제 2차 KPC 개최 심의 안건 #18  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-18 12:53:46 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+9. 2024년도_붙임  (요약)야간경마 행사 추진계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-11 16:38:58 &lt;/Document-Metadata&gt;  문인증 이벤트 등 축제 방문객 경마참…
+10. 2024년도_[붙임2] (본문) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #9  ▸  &lt;Document-Metadata&gt;   제목: 2019   작성자: KRA   마지막 수정자: KRA   작성일: 2019-07-24 15:06:06   수정일: 2024-05-25 09:18:53 &lt;/Document-Metadata&gt;  === Extracted Ima…
+11. 2024년도_붙임2) (경주분류위원회)부의안건 #17  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-18 09:16:43   수정일: 2024-12-28 09:41:41 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+12. 2022년도_(211230)2022_제주경마계획_책자원고(최종수정) #141  ▸  &lt;Document-Metadata&gt;   제목: Ⅱ. 경마 시행 개요   키워드: 
     설명: 
-    마지막 수정자: KRA   작성일: 2005-01-06 17:05:55   수정일: 2021-12-
-[788bbf4ba82b5320] 2022년도_첨부2_2022년 대상경주별 레이스 레이팅 세부 현황(연말 최종) #37  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-14 00:44:46   수정일: 2022-12-16 01:40:17 &lt;/Document-Me
-[83680adc07f09d42] 2022년도_연말연시 대고객 무료입장 행사 시행 결과보고 #7  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-26 11:21:25   수정일: 2022-12-23 09:30:05 &lt;/Document-M
-[929899bce4b8ff3e] 2023년도_첨부2_2023년 대상경주별 레이스 레이팅 세부 현황(연말 최종) #37  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-22 01:15:23   수정일: 2023-12-28 05:16:45 &lt;/Document-Me
-[9e0b5f9c2ae462c6] 2023년도_1등급 경주마 레이팅 현실화_최종 #15  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: user   마지막 수정자: KRA   작성일: 2018-04-17 13:51:47   수정일: 2023-11-26 14:39:29 &lt;/Document-
-[b0fc75f5da7a1c86] 2024년도_(붙임1) 2024년 제주경마방송 운영 계획(안)_요약 (최종) #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-07 09:19:14 &lt;/Document-M
-[b693b284424819ba] 2023년도_붙임_2023년 대상경주 레이스 레이팅 부여결과 보고 #11  ▸  &lt;Document-Metadata&gt;   제목: 2016년 주요 대상경주 Race Rating 부여결과 보고   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-06 09:42:57   수정일:
-[b990e68b5d5d78da] 2023년도_[붙임1] (요약) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2023-11-03 09:16:57   수정일: 2024-05-24 19:48:59 &lt;/Document-M
-[be51e42247813522] 2022년도_시리즈 경주 시행 결과보고 #25  ▸  &lt;Document-Metadata&gt;   제목: 2021년 시리즈 경주 시행 결과보고   작성자: KRA   마지막 수정자: KRA   작성일: 2021-12-15 13:12:50   수정일: 2022-12-17 11
+    마지막 수정자: KRA   작성일: 2005-01-06 17:05:55   수정일: 2021-12-30 13:58:40 &lt;/Document-Metadat…
+13. 2022년도_첨부2_2022년 대상경주별 레이스 레이팅 세부 현황(연말 최종) #37  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-14 00:44:46   수정일: 2022-12-16 01:40:17 &lt;/Document-Metadata&gt;  [Sheet: 대상특별 레이스 레이팅]…
+14. 2022년도_연말연시 대고객 무료입장 행사 시행 결과보고 #7  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-01-26 11:21:25   수정일: 2022-12-23 09:30:05 &lt;/Document-Metadata&gt;  * 대조군 : 무료입장 시행일 전·후…
+15. 2023년도_첨부2_2023년 대상경주별 레이스 레이팅 세부 현황(연말 최종) #37  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-22 01:15:23   수정일: 2023-12-28 05:16:45 &lt;/Document-Metadata&gt;  [Sheet: 대상특별 레이스 레이팅]…
+16. 2023년도_1등급 경주마 레이팅 현실화_최종 #15  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: user   마지막 수정자: KRA   작성일: 2018-04-17 13:51:47   수정일: 2023-11-26 14:39:29 &lt;/Document-Metadata&gt;  - 서울은 “라온더파이터”, 부경은…
+17. 2024년도_(붙임1) 2024년 제주경마방송 운영 계획(안)_요약 (최종) #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-07 09:19:14 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+18. 2023년도_붙임_2023년 대상경주 레이스 레이팅 부여결과 보고 #11  ▸  &lt;Document-Metadata&gt;   제목: 2016년 주요 대상경주 Race Rating 부여결과 보고   작성자: KRA   마지막 수정자: KRA   작성일: 2017-01-06 09:42:57   수정일: 2023-12-28 14:16:06 &lt;/Document…
+19. 2023년도_[붙임1] (요약) 대상경주 우승 기수 「시상대 검량」 추진 계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2023-11-03 09:16:57   수정일: 2024-05-24 19:48:59 &lt;/Document-Metadata&gt;  * 출장로 및 마도를 통한 우승마 대…
+20. 2022년도_시리즈 경주 시행 결과보고 #25  ▸  &lt;Document-Metadata&gt;   제목: 2021년 시리즈 경주 시행 결과보고   작성자: KRA   마지막 수정자: KRA   작성일: 2021-12-15 13:12:50   수정일: 2022-12-17 11:36:04 &lt;/Document-Metadata&gt;  […
 ... +8 more</t>
         </is>
       </c>
@@ -4638,10 +4638,10 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[59854a9e60c7d3ab] 2022년도_(붙임2)재물조사결과내역(전체) #106  ▸  &lt;Document-Metadata&gt;   작성자: KA B &lt;/Document-Metadata&gt;  [Sheet: 전체] [Table Chunk 107/107] | 자산번호 | SAP자산번호 | 자산구분 | 세분류 |
-[6a278de5a7f63982] 2022년도_(붙임1)2022년 정기 재물조사 실시 결과보고 #9  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-23 10:36:27   수정일: 2023-01-19 14:22:42 &lt;/Documen
-[95765c577ef9e336] 2024년도_(붙임1) 2024년 재물조사 시행 결과보고_241227 #15  ▸  &lt;Document-Metadata&gt;   제목: 재물조정   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-12 16:02:40   수정일: 2024-12-27 09:49:24 &lt;/Documen
-[c8ed7811592eac64] 2022년도_(붙임2)재물조사결과내역(전체) #393  ▸  &lt;Document-Metadata&gt;   작성일: 2025-12-05 08:14:00   수정일: 2025-12-05 08:14:00 &lt;/Document-Metadata&gt;  [Page Number: 394]  &lt;tab</t>
+          <t>1. 2022년도_(붙임2)재물조사결과내역(전체) #106  ▸  &lt;Document-Metadata&gt;   작성자: KA B &lt;/Document-Metadata&gt;  [Sheet: 전체] [Table Chunk 107/107] | 자산번호 | SAP자산번호 | 자산구분 | 세분류 | 본부명 | 자산내역 | 취득일자 | 구매금액 | 단가 …
+2. 2022년도_(붙임1)2022년 정기 재물조사 실시 결과보고 #9  ▸  &lt;Document-Metadata&gt;   제목: 2020   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-23 10:36:27   수정일: 2023-01-19 14:22:42 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+3. 2024년도_(붙임1) 2024년 재물조사 시행 결과보고_241227 #15  ▸  &lt;Document-Metadata&gt;   제목: 재물조정   작성자: KRA   마지막 수정자: KRA   작성일: 2024-04-12 16:02:40   수정일: 2024-12-27 09:49:24 &lt;/Document-Metadata&gt;  전 부서    ❍ 조직개편, 인…
+4. 2022년도_(붙임2)재물조사결과내역(전체) #393  ▸  &lt;Document-Metadata&gt;   작성일: 2025-12-05 08:14:00   수정일: 2025-12-05 08:14:00 &lt;/Document-Metadata&gt;  [Page Number: 394]  &lt;table&gt;   &lt;tr&gt;     &lt;th&gt;20220842911…</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -4685,8 +4685,8 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[8390d154aeb39727] 2022년도_붙임 3. 예산전용 세부내역 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-13 05:10:41   수정일: 2023-08-18 04:08:23 &lt;/Document-Metadata&gt;
-[e9e64a316174aed5] 2022년도_[붙임]출전준비소 바닥면 탄성포장 추진안 #1  ▸  &lt;Document-Metadata&gt;   제목: 조명탑 및 감시카메라    작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-26 15:45:00   수정일: 2022-10-15 15:21:52 &lt;</t>
+          <t>1. 2022년도_붙임 3. 예산전용 세부내역 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-08-13 05:10:41   수정일: 2023-08-18 04:08:23 &lt;/Document-Metadata&gt;  [Sheet: 2. 예산산출내역] &lt;table bo…
+2. 2022년도_[붙임]출전준비소 바닥면 탄성포장 추진안 #1  ▸  &lt;Document-Metadata&gt;   제목: 조명탑 및 감시카메라    작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-26 15:45:00   수정일: 2022-10-15 15:21:52 &lt;/Document-Metadata&gt;  2. 바닥 현황 …</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[17bd81589a0131cf] 2024년도_[붙임2] (제24-63호) 직제규정시행세칙 일부 개정(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-15 13:06:07   수정일: 2024-12-13 17:50:27 &lt;/Document-M
-[27dcbb61e82d6f82] 2024년도_과제 및 사업별 담당부서 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-08 02:27:01   수정일: 2024-06-13 05:02:20 &lt;/Document-Metadata&gt;
-[4fbf4a8a7bd53b63] 2023년도_(붙임) D-공원레저 및 지역상생(230222) #50  ▸  &lt;Document-Metadata&gt;   제목: 3   작성자: KRA   마지막 수정자: KRA   작성일: 2021-11-28 15:41:36   수정일: 2023-02-22 14:37:47 &lt;/Document-M
-[a4ed66c59a820e40] 2020년도_(붙임#14) 사업별 조직별 예산 계층구조 #78  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-11 08:44:57   수정일: 2020-03-13 01:24:08 &lt;/Document-Metadata&gt;
-[aa6aff98e2caa723] 2023년도_[붙임2] 2024년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-14 07:46:48   수정일: 2024-01-31 07:29:46 &lt;/Document-Metadata&gt;
-[da8efb3618249a33] 2022년도_[붙임2] 2023년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-02-15 02:28:16   수정일: 2023-02-16 04:38:18 &lt;/Document-Metadata&gt;</t>
+          <t>1. 2024년도_[붙임2] (제24-63호) 직제규정시행세칙 일부 개정(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-11-15 13:06:07   수정일: 2024-12-13 17:50:27 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+2. 2024년도_과제 및 사업별 담당부서 #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-08 02:27:01   수정일: 2024-06-13 05:02:20 &lt;/Document-Metadata&gt;  [Sheet: 과제 및 사업별 담당] [Table …
+3. 2023년도_(붙임) D-공원레저 및 지역상생(230222) #50  ▸  &lt;Document-Metadata&gt;   제목: 3   작성자: KRA   마지막 수정자: KRA   작성일: 2021-11-28 15:41:36   수정일: 2023-02-22 14:37:47 &lt;/Document-Metadata&gt;  [Image:temp/images/h…
+4. 2020년도_(붙임#14) 사업별 조직별 예산 계층구조 #78  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-11 08:44:57   수정일: 2020-03-13 01:24:08 &lt;/Document-Metadata&gt;  [Sheet: 사업별 예산 계층구조] [Table …
+5. 2023년도_[붙임2] 2024년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-14 07:46:48   수정일: 2024-01-31 07:29:46 &lt;/Document-Metadata&gt;  [Sheet: 조직별 예산 계층구조] [Table …
+6. 2022년도_[붙임2] 2023년 사업별 조직별 예산 계층구조 #160  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-02-15 02:28:16   수정일: 2023-02-16 04:38:18 &lt;/Document-Metadata&gt;  [Sheet: 조직별 예산 계층구조] [Table …</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -4779,25 +4779,25 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[012dcbe84f52c595] 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Me
-[0cc573d6922d1cfd] 2024년도_★ 2024년 공정관리 업무추진 계획(안) #5  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-03 15:15:28 &lt;/Document-M
-[157016074626f25d] 2021년도_(별첨1) 연도별 마주 경제적기준(2007_2021) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-20 01:23:19   수정일: 2021-11-26 04:01:22 &lt;/Document-Metadata&gt;
-[1ff851c7c3ee9eb5] 2021년도_(2021) 제 99주년 경마의 날 기념식 시행계획(안)_요약보고 #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2021-05-08 14:10:03 &lt;/Document-Metadat
-[2df376eb9253a430] 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Me
-[5cf871e3bcad9e3b] 2025년도_(붙임3) 2025년 한국마사회 수입 및 지출계획서 #12  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2024-12-19 17:06:39 &lt;/Documen
-[6e8edf545decf5bf] 2021년도_(붙임1) 2021년 더러브렛 마주 운영 개선(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 2021년 마주제도 개선 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-11 15:25:28   수정일: 2021-11-28 09:56:
-[7744ef805224b82a] 2022년도_(제23-14호) 더러브렛등록규정 시행세칙 일부 개정(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2020-05-24 10:48:12   수정일: 2023-04-21 16:37:04 &lt;/Do
-[864c7ea3086114e0] 2021년도_(제21-31호) 경마비위 신고포상금 지급규정 개정_결재(최종)★ #1  ▸  &lt;Document-Metadata&gt;   제목: 임원 징계 규정 제정   작성자: sinyoungpark   마지막 수정자: KRA   작성일: 2020-07-14 15:57:47   수정일: 2021-07-23 17
-[bd4e6e178c18810b] 2022년도_경마시행규정 시행세칙 등 개정(안) #37  ▸  &lt;Document-Metadata&gt;   제목: kjhll   키워드: 
+          <t>1. 2022년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #110  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2022-12-16 01:56:04   수정일: 2022-12-16 02:02:00 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…
+2. 2024년도_★ 2024년 공정관리 업무추진 계획(안) #5  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-02-03 15:15:28 &lt;/Document-Metadata&gt;  등 사전예방활동으로 경마공정성 강화 …
+3. 2021년도_(별첨1) 연도별 마주 경제적기준(2007_2021) #6  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-20 01:23:19   수정일: 2021-11-26 04:01:22 &lt;/Document-Metadata&gt;  [Sheet: 정리본] [Table Chunk 7/…
+4. 2021년도_(2021) 제 99주년 경마의 날 기념식 시행계획(안)_요약보고 #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2021-05-08 14:10:03 &lt;/Document-Metadata&gt;  제 99주년 경마의 날 기념식 시행 (안) 보고…
+5. 2023년도_첨부3_2023년 한국 경주마 국제 레이팅 현황(4등급 이상) #167  ▸  &lt;Document-Metadata&gt;   작성자: Apache POI   마지막 수정자: KRA   작성일: 2023-12-28 04:23:52   수정일: 2023-12-28 04:35:56 &lt;/Document-Metadata&gt;  [Sheet: Int. Rating L…
+6. 2025년도_(붙임3) 2025년 한국마사회 수입 및 지출계획서 #12  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2024-12-19 17:06:39 &lt;/Document-Metadata&gt;  훈), 예산담당사원(강현석)  …
+7. 2021년도_(붙임1) 2021년 더러브렛 마주 운영 개선(안) #11  ▸  &lt;Document-Metadata&gt;   제목: 2021년 마주제도 개선 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-06-11 15:25:28   수정일: 2021-11-28 09:56:00 &lt;/Document-Metadata&gt;  0대 이상…
+8. 2022년도_(제23-14호) 더러브렛등록규정 시행세칙 일부 개정(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2020-05-24 10:48:12   수정일: 2023-04-21 16:37:04 &lt;/Document-Metadata&gt;  &lt;table borde…
+9. 2021년도_(제21-31호) 경마비위 신고포상금 지급규정 개정_결재(최종)★ #1  ▸  &lt;Document-Metadata&gt;   제목: 임원 징계 규정 제정   작성자: sinyoungpark   마지막 수정자: KRA   작성일: 2020-07-14 15:57:47   수정일: 2021-07-23 17:57:06 &lt;/Document-Metadata&gt;  &lt;…
+10. 2022년도_경마시행규정 시행세칙 등 개정(안) #37  ▸  &lt;Document-Metadata&gt;   제목: kjhll   키워드: 
     설명: 
-    마지막 수정자: KRA   작성일: 2006-01-20 14:28:49   수정일: 2023-02-25 17:
-[c142c30f937d4868] 2020년도_[붙임1] (요약) 2020년 K-Nicks를 활용한 국내산마 미국 수출 지원계획(안) #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-04-13 11:03:16   수정일: 2020-06-04 16:21:38 &lt;/Document-Metadata&gt;
-[c1ebd6c13900514d] 2021년도_(붙임2) 경주퇴역마 복지 가이드라인(최종안) #3  ▸  &lt;Document-Metadata&gt;   제목: 경주퇴역마 가이드라인 제정 관련   작성자: KRA   마지막 수정자: KRA   작성일: 2021-08-13 09:51:05   수정일: 2021-12-04 10:33
-[d91964b859494daf] 2021년도_(붙임3)_2021년도 수입 및 지출 계획서 #14  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2020-12-18 18:13:07 &lt;/Documen
-[da80398d5e7b1d5b] 2021년도_2020 한국경마 대국민 인식조사 설문지 #15  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-02-26 15:05:29   수정일: 2021-02-26 15:06:19 &lt;/Document-Metadata&gt;
-[de08827cf2920b82] 2024년도_(요약) 2024년 서울경마공원 경주마 재활지원 프로그램 운영계획 #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-23 17:05:09 &lt;/Document-M
-[f960b0c32b20eee5] 2024년도_(요약) 2024년 서울경마공원 경주마 재활지원 프로그램 운영계획 #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-23 17:05:09 &lt;/Document-M
-[fe8f39c7158239fe] 2023년도_2023 가을승마주간 시행 기본계획(안) #20  ▸  &lt;Document-Metadata&gt;   제목: 서울 경마공원에서    작성자: KRA   마지막 수정자: KRA   작성일: 2023-10-06 08:45:07   수정일: 2023-10-14 18:38:53 &lt;/D</t>
+    마지막 수정자: KRA   작성일: 2006-01-20 14:28:49   수정일: 2023-02-25 17:22:06 &lt;/Document-Metadata&gt;  &lt;t…
+11. 2020년도_[붙임1] (요약) 2020년 K-Nicks를 활용한 국내산마 미국 수출 지원계획(안) #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-04-13 11:03:16   수정일: 2020-06-04 16:21:38 &lt;/Document-Metadata&gt;  농가 홍보    말등록원 : 수출시 수출증명서 발행…
+12. 2021년도_(붙임2) 경주퇴역마 복지 가이드라인(최종안) #3  ▸  &lt;Document-Metadata&gt;   제목: 경주퇴역마 가이드라인 제정 관련   작성자: KRA   마지막 수정자: KRA   작성일: 2021-08-13 09:51:05   수정일: 2021-12-04 10:33:13 &lt;/Document-Metadata&gt;  라. 말…
+13. 2021년도_(붙임3)_2021년도 수입 및 지출 계획서 #14  ▸  &lt;Document-Metadata&gt;   제목: 2018   작성자: KRA   마지막 수정자: KRA   작성일: 2018-12-08 16:36:27   수정일: 2020-12-18 18:13:07 &lt;/Document-Metadata&gt;  재원), 예산담당대리(권오경) …
+14. 2021년도_2020 한국경마 대국민 인식조사 설문지 #15  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-02-26 15:05:29   수정일: 2021-02-26 15:06:19 &lt;/Document-Metadata&gt;  의 결혼상태는 어떻습니까?   	ཧĀ	1. 미혼  …
+15. 2024년도_(요약) 2024년 서울경마공원 경주마 재활지원 프로그램 운영계획 #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-23 17:05:09 &lt;/Document-Metadata&gt;  서울경마공원  2024년 경주마 재활…
+16. 2024년도_(요약) 2024년 서울경마공원 경주마 재활지원 프로그램 운영계획 #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-03-23 17:05:09 &lt;/Document-Metadata&gt;  서울경마공원  2024년 경주마 재활…
+17. 2023년도_2023 가을승마주간 시행 기본계획(안) #20  ▸  &lt;Document-Metadata&gt;   제목: 서울 경마공원에서    작성자: KRA   마지막 수정자: KRA   작성일: 2023-10-06 08:45:07   수정일: 2023-10-14 18:38:53 &lt;/Document-Metadata&gt;  &lt;table bord…</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -4854,18 +4854,18 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[23f259fe9f9c25d9] 2020년도_200828_언택트발매추진단 하반기 사업계획 및 예산 #4  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-21 12:13:34   수정일: 2020-08-28 13:15:23 &lt;/Document-M
-[24413d0baba3f505] 2020년도_(붙임)'20 이용자보호 현업과제 운영계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제도 확산   작성자: KRA   마지막 수정자: KRA   작성일: 2020-06-12 15:43:26   수정일: 2020-07-25 17:48:38 &lt;/Docume
-[3b6b26357ad2ce21] 2020년도_(요약) 2020년 이용자보호 추진계획 보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-21 13:18:29 &lt;/Document-M
-[594cc15f51062da3] 2023년도_[붙임] 2023년 ESG경영 추진계획(안)_최종 #37  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-05-27 10:36:47 &lt;/Document-Metadata&gt;
-[5d0dd8502b5a0cb8] 2020년도_(본문) 20년 이용자보호 액션플랜 수립계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 제목    작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-16 09:57:57   수정일: 2020-02-09 15:46:56 &lt;/Document
-[853bed249201f55c] 2020년도_[붙임1](요약)온라인 고도화 및 미래대응체계구축 기본계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-15 09:26:37   수정일: 2020-03-28 14:50:47 &lt;/Documen
-[93494a02861846af] 2023년도_붙임_2023년 사감위 건전화평가 관리계획(안)_230617_결재 #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-08 17:12:29   수정일: 2023-06-17 15:12:03 &lt;/Document-Metadata&gt;
-[957fa34075bbf580] 2021년도_(요약) `21년경마 건전화 추진 계획(안) #4  ▸  &lt;Document-Metadata&gt;   제목: CEO지시사항 추진과제 입력 매뉴얼   작성자: kra   마지막 수정자: KRA   작성일: 2014-03-29 09:25:36   수정일: 2021-07-23 14:
-[9c30b7128e4e1947] 2020년도_(별첨) 참고_과제별중장기실행계획('19년) #0  ▸  &lt;Document-Metadata&gt;   제목: □ 과제개요   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-09 14:11:10   수정일: 2020-02-09 14:46:38 &lt;/Docum
-[c1967d59910a20e6] 2021년도_(본문) `21년 경마 건전화 추진 계획(안) #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2015-11-06 10:21:54   수정일: 2021-07-23 14:20:18 &lt;/Document-Metadata&gt;
-[cc2b1d26273fcdab] 2024년도_붙임_2024년 사행산업사업자 건전화평가 관리계획(안)_240518_결재 #24  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-08 17:12:29   수정일: 2024-05-18 17:43:16 &lt;/Document-Metadata&gt;
-[d4d20ca93dfcd728] 2020년도_(본문) 2020년 이용자보호 추진계획 #15  ▸  &lt;Document-Metadata&gt;   제목: 회의자료    작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-19 16:10:55   수정일: 2020-03-21 10:39:32 &lt;/Docume</t>
+          <t>1. 2020년도_200828_언택트발매추진단 하반기 사업계획 및 예산 #4  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2020-07-21 12:13:34   수정일: 2020-08-28 13:15:23 &lt;/Document-Metadata&gt;  및 말산업 생태계 보존     (이용…
+2. 2020년도_(붙임)'20 이용자보호 현업과제 운영계획 #7  ▸  &lt;Document-Metadata&gt;   제목: 제도 확산   작성자: KRA   마지막 수정자: KRA   작성일: 2020-06-12 15:43:26   수정일: 2020-07-25 17:48:38 &lt;/Document-Metadata&gt;  가. 추진절차  &lt;table …
+3. 2020년도_(요약) 2020년 이용자보호 추진계획 보고 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-03-21 13:18:29 &lt;/Document-Metadata&gt;  * 세부 추진계획은 과제별로 별도 수…
+4. 2023년도_[붙임] 2023년 ESG경영 추진계획(안)_최종 #37  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2023-01-28 11:07:34   수정일: 2023-05-27 10:36:47 &lt;/Document-Metadata&gt;  * ESG 추진과제 관련 현안 발생 시 별도 보고 …
+5. 2020년도_(본문) 20년 이용자보호 액션플랜 수립계획(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 제목    작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-16 09:57:57   수정일: 2020-02-09 15:46:56 &lt;/Document-Metadata&gt;  [Image:temp/images…
+6. 2020년도_[붙임1](요약)온라인 고도화 및 미래대응체계구축 기본계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 보고자    작성자: KRA   마지막 수정자: KRA   작성일: 2020-03-15 09:26:37   수정일: 2020-03-28 14:50:47 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+7. 2023년도_붙임_2023년 사감위 건전화평가 관리계획(안)_230617_결재 #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-08 17:12:29   수정일: 2023-06-17 15:12:03 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+8. 2021년도_(요약) `21년경마 건전화 추진 계획(안) #4  ▸  &lt;Document-Metadata&gt;   제목: CEO지시사항 추진과제 입력 매뉴얼   작성자: kra   마지막 수정자: KRA   작성일: 2014-03-29 09:25:36   수정일: 2021-07-23 14:20:55 &lt;/Document-Metadata&gt;  보안…
+9. 2020년도_(별첨) 참고_과제별중장기실행계획('19년) #0  ▸  &lt;Document-Metadata&gt;   제목: □ 과제개요   작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-09 14:11:10   수정일: 2020-02-09 14:46:38 &lt;/Document-Metadata&gt;  &lt;table border='…
+10. 2021년도_(본문) `21년 경마 건전화 추진 계획(안) #1  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2015-11-06 10:21:54   수정일: 2021-07-23 14:20:18 &lt;/Document-Metadata&gt;  * `21년 건전화 평가 편람 개요 : 4개 부문,…
+11. 2024년도_붙임_2024년 사행산업사업자 건전화평가 관리계획(안)_240518_결재 #24  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2022-06-08 17:12:29   수정일: 2024-05-18 17:43:16 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+12. 2020년도_(본문) 2020년 이용자보호 추진계획 #15  ▸  &lt;Document-Metadata&gt;   제목: 회의자료    작성자: KRA   마지막 수정자: KRA   작성일: 2020-02-19 16:10:55   수정일: 2020-03-21 10:39:32 &lt;/Document-Metadata&gt;  (고객보호부) 과제 총괄 관리…</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -4917,30 +4917,30 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[03e46e426c5e0a40] 2022년도_(붙임1) 인사규정시행세칙 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:10:39 &lt;/Document-Metadata&gt;
-[0fdd2b845b06532f] 2024년도_2024년 기부금 지원공모사업(안) #14  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2015-10-08 19:55:17   수정일: 2024-08-10 11:00:13 &lt;/Document-M
-[1002c0855b631621] 2022년도_한국마사회 ESG경영부 2022년 인권경영 이행실적 보고서 견적서 #1  ▸  &lt;Document-Metadata&gt;   작성자: Administrator   마지막 수정자: 이주훈   작성일: 2012-01-19 08:40:24   수정일: 2023-06-18 09:36:47 &lt;/Document
-[2520e4f72ad580ae] 2022년도_(제23-11호) 인권경영 실행지침 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-04 09:10:19   수정일: 2023-04-23 10:51:13 &lt;/Do
-[27e3f288a3dda838] 2024년도_지사, 문화센터 홈페이지 개편 계획(안)_240526(수정) #11  ▸  &lt;Document-Metadata&gt;   제목: □ 통합신고센터 운영개선을 통해 불법경마 신고접수 전문인력 양성   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-24 13:51:43   수정일
-[320953785300baf0] 2023년도_(붙임4) 위촉직관리지침 일부 개정(안) #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:09 &lt;/Document-Metadata&gt;
-[329af5c7de78350a] 2024년도_(붙임) 2024년 인권경영 기본계획(안)_240414★ #2  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2024-04-16 16:56:55 &lt;/Documen
-[3a729c75753c7cf2] 2024년도_붙임1. 인권경영위원회 회의자료 #15  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-10-13 14:35:36   수정일: 2024-11-27 13:38:05 &lt;/Document-Metadata&gt;
-[3b38d7e7d3da74e2] 2024년도_(요약) 2024년 인권경영 기본계획(안)  ▸  2024년도_(요약) 2024년 인권경영 기본계획(안)
-[455c41ea7d950aff] 2020년도_불법경마사이트 신고 활성화를 위한 고객신고 제도 분석 및 운영 개선(안) #9  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-04 16:43:55   수정일: 2020-01-19 13:58:22 &lt;/Document-M
-[475035a5d7c43233] 2023년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;
-[499f2103edc5d6e1] 2021년도_(본문) 2021년 인권경영 기본계획 #30  ▸  &lt;Document-Metadata&gt;   제목: 2021년도 인권경영 추진계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-05-14 10:44:55   수정일: 2021-05-29 15:39:
-[4cab49368cf80ad5] 2023년도_(결재) 2023년 인권경영 기본계획(최종) #1  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2023-04-13 17:11:11 &lt;/Documen
-[4e67027b23247ea7] 2022년도_[붙임] 「불법경마 신고포상금 지급 등에 관한 규정」 일부 개정안 #0  ▸  &lt;Document-Metadata&gt;   제목: 경주정보 불법 송출   작성자: KRA   마지막 수정자: KRA   작성일: 2022-07-09 19:23:20   수정일: 2022-12-04 15:24:16 &lt;/D
-[55ab962e1bccc09b] 2022년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;
-[6c8917aa77bbade5] 2021년도_(요약) 2021년 인권경영 기본계획 #8  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2021-05-29 15:
-[7137b1d9495ea540] 2024년도_붙임1. 인권경영실행지침 일부 개정(안)_수정(241012) #15  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2023-11-01 14:09:00   수정일: 2024-10-12 16:56:29 &lt;/Document-M
-[722ac78a66cc46c2] 2024년도_[붙임1] 601. 취업규칙 전문(20241214)-제36차 개정 #34  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
+          <t>1. 2022년도_(붙임1) 인사규정시행세칙 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:10:39 &lt;/Document-Metadata&gt;  ※ 작성방법 : 점검결과에 ‘적정’ 또는 ‘부적정’…
+2. 2024년도_2024년 기부금 지원공모사업(안) #14  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2015-10-08 19:55:17   수정일: 2024-08-10 11:00:13 &lt;/Document-Metadata&gt;  6) 추진일정    - 프로그램별 세…
+3. 2022년도_한국마사회 ESG경영부 2022년 인권경영 이행실적 보고서 견적서 #1  ▸  &lt;Document-Metadata&gt;   작성자: Administrator   마지막 수정자: 이주훈   작성일: 2012-01-19 08:40:24   수정일: 2023-06-18 09:36:47 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt;…
+4. 2022년도_(제23-11호) 인권경영 실행지침 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   제목: 신명조 17 pt   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-04 09:10:19   수정일: 2023-04-23 10:51:13 &lt;/Document-Metadata&gt;  동과 아동노동도 허용하…
+5. 2024년도_지사, 문화센터 홈페이지 개편 계획(안)_240526(수정) #11  ▸  &lt;Document-Metadata&gt;   제목: □ 통합신고센터 운영개선을 통해 불법경마 신고접수 전문인력 양성   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-24 13:51:43   수정일: 2024-05-26 09:42:09 &lt;/Docume…
+6. 2023년도_(붙임4) 위촉직관리지침 일부 개정(안) #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:09 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+7. 2024년도_(붙임) 2024년 인권경영 기본계획(안)_240414★ #2  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2024-04-16 16:56:55 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+8. 2024년도_붙임1. 인권경영위원회 회의자료 #15  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-10-13 14:35:36   수정일: 2024-11-27 13:38:05 &lt;/Document-Metadata&gt;  ○ 교육, 강습 및 기타사업 분야  &lt;table b…
+9. 2024년도_(요약) 2024년 인권경영 기본계획(안)  ▸  2024년도_(요약) 2024년 인권경영 기본계획(안)
+10. 2020년도_불법경마사이트 신고 활성화를 위한 고객신고 제도 분석 및 운영 개선(안) #9  ▸  &lt;Document-Metadata&gt;   제목: Ⅰ   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-04 16:43:55   수정일: 2020-01-19 13:58:22 &lt;/Document-Metadata&gt;  시 (2분기)     ※ 불법경마 대…
+11. 2023년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;  년    월    일   &lt;table border=…
+12. 2021년도_(본문) 2021년 인권경영 기본계획 #30  ▸  &lt;Document-Metadata&gt;   제목: 2021년도 인권경영 추진계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-05-14 10:44:55   수정일: 2021-05-29 15:39:40 &lt;/Document-Metadata&gt;  === E…
+13. 2023년도_(결재) 2023년 인권경영 기본계획(최종) #1  ▸  &lt;Document-Metadata&gt;   제목: 추진배경   작성자: KRA   마지막 수정자: KRA   작성일: 2023-04-05 11:22:01   수정일: 2023-04-13 17:11:11 &lt;/Document-Metadata&gt;  8.)        * 경영평가…
+14. 2022년도_[붙임] 「불법경마 신고포상금 지급 등에 관한 규정」 일부 개정안 #0  ▸  &lt;Document-Metadata&gt;   제목: 경주정보 불법 송출   작성자: KRA   마지막 수정자: KRA   작성일: 2022-07-09 19:23:20   수정일: 2022-12-04 15:24:16 &lt;/Document-Metadata&gt;  『불법경마 신고포상금…
+15. 2022년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;  년    월    일   &lt;table border=…
+16. 2021년도_(요약) 2021년 인권경영 기본계획 #8  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2021-05-29 15:41:30 &lt;/Document-Metadata&gt;  &lt;t…
+17. 2024년도_붙임1. 인권경영실행지침 일부 개정(안)_수정(241012) #15  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2023-11-01 14:09:00   수정일: 2024-10-12 16:56:29 &lt;/Document-Metadata&gt;  20  .   .     인권경영책임…
+18. 2024년도_[붙임1] 601. 취업규칙 전문(20241214)-제36차 개정 #34  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
     설명: 
-    마지막 수정자: KRA   작성일: 2006-03-14 16:07:44   수정일: 2024-12-15 09:
-[725ae7e3f94266ed] 2024년도_붙임1. ‘24년 제1차 인권경영위원회 개최계획(안) #0  ▸  &lt;Document-Metadata&gt;   제목: 개최개요   작성자: KRA   마지막 수정자: KRA   작성일: 2023-12-06 16:00:46   수정일: 2024-08-10 14:26:38 &lt;/Documen
-[7610ecb82f1d71e2] 2024년도_(전문)성희롱·성폭력_ 직장내 괴롭힘 및 스토킹 예방지침(241228)최종 #22  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
+    마지막 수정자: KRA   작성일: 2006-03-14 16:07:44   수정일: 2024-12-15 09:17:04 &lt;/Document-Metadata&gt;  [별…
+19. 2024년도_붙임1. ‘24년 제1차 인권경영위원회 개최계획(안) #0  ▸  &lt;Document-Metadata&gt;   제목: 개최개요   작성자: KRA   마지막 수정자: KRA   작성일: 2023-12-06 16:00:46   수정일: 2024-08-10 14:26:38 &lt;/Document-Metadata&gt;  ‘24년 제1차 인권경영위원회 …
+20. 2024년도_(전문)성희롱·성폭력_ 직장내 괴롭힘 및 스토킹 예방지침(241228)최종 #22  ▸  &lt;Document-Metadata&gt;   제목: 인사,후생   키워드: 
     설명: 
-    마지막 수정자: KRA   작성일: 2006-03-14 16:07:44   수정일: 2024-12-28 09:
+    마지막 수정자: KRA   작성일: 2006-03-14 16:07:44   수정일: 2024-12-28 09:23:18 &lt;/Document-Metadata&gt;  [별…
 ... +30 more</t>
         </is>
       </c>
@@ -5031,19 +5031,19 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[1dd7a41b6d49067a] 2020년도_붙임_2_2020년 도심승마체험 시행계획(본문, 최종) #55  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-09 13:50:33   수정일: 2020-03-11 10:31:15 &lt;/Document-M
-[230b3c89a0f6cfdc] 2023년도_붙임 1. 2023년 학교체육 승마 시범사업 운영계획(안) #35  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-11-04 14:57:12   수정일: 2022-12-02 16:28:09 &lt;/Document-Metadata&gt;
-[2cbdb440161c0502] 2024년도_2024년 제주경마공원 승마체험장 및 관상마체험장 운영계획 #17  ▸  &lt;Document-Metadata&gt;   제목: 2014   마지막 수정자: KRA   작성일: 2014-02-07 09:49:57   수정일: 2024-02-28 11:03:22 &lt;/Document-Metadata&gt;
-[345beb807d95ba70] 2020년도_★(결재) 2020 사회공익힐링 승마 사업 기본 운영 계획 #5  ▸  &lt;Document-Metadata&gt;   제목: 2019 전국민 승마체험 사업 기본계획   작성자: user   마지막 수정자: KRA   작성일: 2019-02-15 13:56:48   수정일: 2020-02-26
-[3811d5c616420fc2] 2024년도_240307 2024 유소년 승마지원 기본계획(요약)(최최종) #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-17 13:38:28   수정일: 2024-03-08 14:41:05 &lt;/Document-M
-[49833f0ed56ba434] 2023년도_제18회 제주마 축제 공고문 및 제안서 #37  ▸  &lt;Document-Metadata&gt;   제목: g   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-01 15:17:22   수정일: 2023-08-20 16:04:43 &lt;/Document-M
-[5619e37e7ee1470d] 2024년도_(양식) 말산업육성지원사업 추진실적 #2  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-28 14:58:32   수정일: 2024-06-13 14:38:26 &lt;/Document-Metadata&gt;
-[68c173524cf22c47] 2020년도_붙임_1_2020년 도심승마체험 시행계획(요약, 최종) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-03-07 18:01:46 &lt;/Document-Metadat
-[7b5af8d8a80073c5] 2023년도_[요약] 2023년 힐링승마 지원사업 추진 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-03-09 14:06:41 &lt;/Document-M
-[affde3091ecbe443] 2024년도_제주마축제 홍보 계획_최종 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-31 19:39:40 &lt;/Document-M
-[c3b5928050f2e9aa] 2024년도_(붙임1) 2024년 도심공원 승마체험 운영계획 변경(안) #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-07 14:26:11   수정일: 2024-06-07 17:52:12 &lt;/Document-M
-[c4f8c5320a9a943c] 2023년도_제18회 제주마 축제 시행계획(안) #26  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2023-08-20 16:19:01 &lt;/Docume
-[edf8fe17a083f95c] 2024년도_[붙임#1] (요약본) 2024년 힐링승마 지원사업 추진 계획(안)_ver2 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-02-22 19:09:53 &lt;/Document-M</t>
+          <t>1. 2020년도_붙임_2_2020년 도심승마체험 시행계획(본문, 최종) #55  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2019-01-09 13:50:33   수정일: 2020-03-11 10:31:15 &lt;/Document-Metadata&gt;  === Extracted Images…
+2. 2023년도_붙임 1. 2023년 학교체육 승마 시범사업 운영계획(안) #35  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2021-11-04 14:57:12   수정일: 2022-12-02 16:28:09 &lt;/Document-Metadata&gt;  * 학교별 전·출입 인원을 감안하여 5% 범위에서 …
+3. 2024년도_2024년 제주경마공원 승마체험장 및 관상마체험장 운영계획 #17  ▸  &lt;Document-Metadata&gt;   제목: 2014   마지막 수정자: KRA   작성일: 2014-02-07 09:49:57   수정일: 2024-02-28 11:03:22 &lt;/Document-Metadata&gt;  【붙임 2】  관상마사 시설현황     주요시설  …
+4. 2020년도_★(결재) 2020 사회공익힐링 승마 사업 기본 운영 계획 #5  ▸  &lt;Document-Metadata&gt;   제목: 2019 전국민 승마체험 사업 기본계획   작성자: user   마지막 수정자: KRA   작성일: 2019-02-15 13:56:48   수정일: 2020-02-26 18:10:51 &lt;/Document-Metadata&gt; …
+5. 2024년도_240307 2024 유소년 승마지원 기본계획(요약)(최최종) #0  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2024-01-17 13:38:28   수정일: 2024-03-08 14:41:05 &lt;/Document-Metadata&gt;  2024 유소년 승마지원 기본계획(안…
+6. 2023년도_제18회 제주마 축제 공고문 및 제안서 #37  ▸  &lt;Document-Metadata&gt;   제목: g   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-01 15:17:22   수정일: 2023-08-20 16:04:43 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+7. 2024년도_(양식) 말산업육성지원사업 추진실적 #2  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-02-28 14:58:32   수정일: 2024-06-13 14:38:26 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+8. 2020년도_붙임_1_2020년 도심승마체험 시행계획(요약, 최종) #0  ▸  &lt;Document-Metadata&gt;   작성자: Owner   마지막 수정자: KRA   작성일: 2008-04-15 17:25:03   수정일: 2020-03-07 18:01:46 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;t…
+9. 2023년도_[요약] 2023년 힐링승마 지원사업 추진 계획(안) #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2023-03-09 14:06:41 &lt;/Document-Metadata&gt;  ※ 출석율 및 신청취소 등을 감안하여…
+10. 2024년도_제주마축제 홍보 계획_최종 #3  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-08-31 19:39:40 &lt;/Document-Metadata&gt;  다양한 홍보 및 광고로 사전 행사 분…
+11. 2024년도_(붙임1) 2024년 도심공원 승마체험 운영계획 변경(안) #1  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2024-06-07 14:26:11   수정일: 2024-06-07 17:52:12 &lt;/Document-Metadata&gt;  * 도심승마체험 가능 장소에 직접 방…
+12. 2023년도_제18회 제주마 축제 시행계획(안) #26  ▸  &lt;Document-Metadata&gt;   제목: 외부 환경   작성자: KRA   마지막 수정자: KRA   작성일: 2017-11-14 10:11:04   수정일: 2023-08-20 16:19:01 &lt;/Document-Metadata&gt;  약합니다.    1. 본인은“…
+13. 2024년도_[붙임#1] (요약본) 2024년 힐링승마 지원사업 추진 계획(안)_ver2 #3  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2024-02-22 19:09:53 &lt;/Document-Metadata&gt;  5. 추진일정  &lt;table bord…</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -5096,26 +5096,26 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[03e46e426c5e0a40] 2022년도_(붙임1) 인사규정시행세칙 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:10:39 &lt;/Document-Metadata&gt;
-[06ea8eb0c6498c61] 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-M
-[0cc6e308b2160025] 2024년도_(요약) 2024년 선수단(유도탁구) 운영 계획_240427 #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-19 14:09:35   수정일: 2024-04-27 10:24:26 &lt;/Document-Metadata&gt;
-[0fdd2b845b06532f] 2024년도_2024년 기부금 지원공모사업(안) #14  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2015-10-08 19:55:17   수정일: 2024-08-10 11:00:13 &lt;/Document-M
-[1ab7e770624479a7] 2024년도_(입찰공고문) 스마트 조교정보시스템 구축 #9  ▸  &lt;Document-Metadata&gt;   제목: 입찰공고문   마지막 수정자: KRA   작성일: 2007-05-20 11:05:36   수정일: 2024-05-10 17:36:20 &lt;/Document-Metadata
-[210e0e2db641965a] 2020년도_[붙임 1] 2020년 재활승마 활성화 지원 시범사업 계획(안_요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 말산업육성본부   작성자: KRA   마지막 수정자: KRA   작성일: 2017-05-24 17:59:41   수정일: 2020-08-07 15:31:04 &lt;/Docu
-[27325f8e49d559f4] 2020년도_(본문) 2020년도 내부경영평가제도 개선(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-22 09:53:12 &lt;/Documen
-[2a67e1073fe83029] 2022년도_2022 힐링승마 지원사업 운영 결과보고_221222 #25  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-08-06 09:18:55   수정일: 2022-12-22 18:09:26 &lt;/Document-Metadata&gt;
-[2c473c597114e075] 2024년도_(요약) 2024년 윤리경영 추진계획(안) (1) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-05-30 11:08:03 &lt;/Document-M
-[2ffc5467d8f17d86] 2020년도_(본문) 2020년 한국마사회 지식경영 운영계획(안)(200417) #19  ▸  &lt;Document-Metadata&gt;   제목: 2017년 지식경영 운영계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-13 15:38:51   수정일: 2020-04-17 10:22:3
-[320953785300baf0] 2023년도_(붙임4) 위촉직관리지침 일부 개정(안) #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:09 &lt;/Document-Metadata&gt;
-[363c897a38703bf5] 2023년도_[요약]한국마사회 CEO·임차인 「청·심·환 간담회」 결과보고 #2  ▸  &lt;Document-Metadata&gt;   제목: □ 편의점 물건   작성자: KRA   마지막 수정자: KRA   작성일: 2022-12-27 14:49:26   수정일: 2023-09-07 14:18:28 &lt;/Doc
-[386c3d238d9e12b0] 2021년도_(요약) 2021 사회공익 힐링승마 사업 결과보고 #4  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-23 17:48:23 &lt;/Document-M
-[40122ffcb05effea] 2020년도_★(요약) 2020 사회공익힐링 승마 사업 기본 운영 계획 #10  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-04 13:13:33   수정일: 2020-02-26 16:19:50 &lt;/Document-Metadata&gt;
-[470d301f2c963cc9] 2020년도_(요약) 2020년 한국마사회 지식경영 운영계획(안)(200417) #1  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2020-04-17 09:
-[475035a5d7c43233] 2023년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;
-[49833f0ed56ba434] 2023년도_제18회 제주마 축제 공고문 및 제안서 #37  ▸  &lt;Document-Metadata&gt;   제목: g   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-01 15:17:22   수정일: 2023-08-20 16:04:43 &lt;/Document-M
-[499f2103edc5d6e1] 2021년도_(본문) 2021년 인권경영 기본계획 #30  ▸  &lt;Document-Metadata&gt;   제목: 2021년도 인권경영 추진계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-05-14 10:44:55   수정일: 2021-05-29 15:39:
-[4b93e74ded9f99c1] 2020년도_2020년 지사 맞춤형 사회적가치 실현  추진 계획(안)) #39  ▸  &lt;Document-Metadata&gt;   제목: 일자리 창출 중장기 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-09-12 12:21:29   수정일: 2020-03-15 17:49:55
-[4bd81a5d3f7d0759] 2024년도_2024년 청심환 간담회 시행 계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: □    작성자: KRA   마지막 수정자: KRA   작성일: 2023-07-13 17:49:14   수정일: 2024-07-20 15:25:58 &lt;/Document-
+          <t>1. 2022년도_(붙임1) 인사규정시행세칙 일부 개정(안) #4  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:10:39 &lt;/Document-Metadata&gt;  ※ 작성방법 : 점검결과에 ‘적정’ 또는 ‘부적정’…
+2. 2020년도_(요약) 2020년도 내부경영평가제도 개선(안) #2  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2020-02-22 09:53:35 &lt;/Document-Metadata&gt;  가와 사업성과평가 통합    ◦ (차…
+3. 2024년도_(요약) 2024년 선수단(유도탁구) 운영 계획_240427 #3  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2024-03-19 14:09:35   수정일: 2024-04-27 10:24:26 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+4. 2024년도_2024년 기부금 지원공모사업(안) #14  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2015-10-08 19:55:17   수정일: 2024-08-10 11:00:13 &lt;/Document-Metadata&gt;  6) 추진일정    - 프로그램별 세…
+5. 2024년도_(입찰공고문) 스마트 조교정보시스템 구축 #9  ▸  &lt;Document-Metadata&gt;   제목: 입찰공고문   마지막 수정자: KRA   작성일: 2007-05-20 11:05:36   수정일: 2024-05-10 17:36:20 &lt;/Document-Metadata&gt;  제출서류는 계약서에 특별히 명기하는 내용 외에는 …
+6. 2020년도_[붙임 1] 2020년 재활승마 활성화 지원 시범사업 계획(안_요약) #0  ▸  &lt;Document-Metadata&gt;   제목: 말산업육성본부   작성자: KRA   마지막 수정자: KRA   작성일: 2017-05-24 17:59:41   수정일: 2020-08-07 15:31:04 &lt;/Document-Metadata&gt;  [Image:temp/im…
+7. 2020년도_(본문) 2020년도 내부경영평가제도 개선(안) #21  ▸  &lt;Document-Metadata&gt;   제목: 2015   작성자: KRA   마지막 수정자: KRA   작성일: 2016-02-11 13:58:39   수정일: 2020-02-22 09:53:12 &lt;/Document-Metadata&gt;  &lt;table border='1'…
+8. 2022년도_2022 힐링승마 지원사업 운영 결과보고_221222 #25  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2019-08-06 09:18:55   수정일: 2022-12-22 18:09:26 &lt;/Document-Metadata&gt;  &lt; 하반기 현장점검 결과 및 의견 &gt;  &lt;table…
+9. 2024년도_(요약) 2024년 윤리경영 추진계획(안) (1) #4  ▸  &lt;Document-Metadata&gt;   제목: 1   작성자: KRA   마지막 수정자: KRA   작성일: 2022-02-27 09:21:34   수정일: 2024-05-30 11:08:03 &lt;/Document-Metadata&gt;  □ CEO 주도의 윤리경영 활동 및 …
+10. 2020년도_(본문) 2020년 한국마사회 지식경영 운영계획(안)(200417) #19  ▸  &lt;Document-Metadata&gt;   제목: 2017년 지식경영 운영계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-03-13 15:38:51   수정일: 2020-04-17 10:22:34 &lt;/Document-Metadata&gt;  부서 심사 …
+11. 2023년도_(붙임4) 위촉직관리지침 일부 개정(안) #5  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:09 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+12. 2023년도_[요약]한국마사회 CEO·임차인 「청·심·환 간담회」 결과보고 #2  ▸  &lt;Document-Metadata&gt;   제목: □ 편의점 물건   작성자: KRA   마지막 수정자: KRA   작성일: 2022-12-27 14:49:26   수정일: 2023-09-07 14:18:28 &lt;/Document-Metadata&gt;  &lt;table border…
+13. 2021년도_(요약) 2021 사회공익 힐링승마 사업 결과보고 #4  ▸  &lt;Document-Metadata&gt;   제목: 22008년도 추경예산   마지막 수정자: KRA   작성일: 2008-06-24 14:14:18   수정일: 2021-12-23 17:48:23 &lt;/Document-Metadata&gt;  * 스트레스 감소 인원 대상 강습 전…
+14. 2020년도_★(요약) 2020 사회공익힐링 승마 사업 기본 운영 계획 #10  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-01-04 13:13:33   수정일: 2020-02-26 16:19:50 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;tr&gt; &lt;td&gt;…
+15. 2020년도_(요약) 2020년 한국마사회 지식경영 운영계획(안)(200417) #1  ▸  &lt;Document-Metadata&gt;   제목: 제1차 청렴옴부즈만 회의 개최 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2010-05-16 09:55:27   수정일: 2020-04-17 09:40:22 &lt;/Document-Metadata&gt;  3.…
+16. 2023년도_(붙임3) 전임직관리지침 일부 개정(안) #7  ▸  &lt;Document-Metadata&gt;   작성자: KRA   마지막 수정자: KRA   작성일: 2020-04-16 10:59:14   수정일: 2023-09-08 11:11:16 &lt;/Document-Metadata&gt;  년    월    일   &lt;table border=…
+17. 2023년도_제18회 제주마 축제 공고문 및 제안서 #37  ▸  &lt;Document-Metadata&gt;   제목: g   작성자: KRA   마지막 수정자: KRA   작성일: 2016-07-01 15:17:22   수정일: 2023-08-20 16:04:43 &lt;/Document-Metadata&gt;  &lt;table border='1'&gt; &lt;…
+18. 2021년도_(본문) 2021년 인권경영 기본계획 #30  ▸  &lt;Document-Metadata&gt;   제목: 2021년도 인권경영 추진계획   작성자: KRA   마지막 수정자: KRA   작성일: 2021-05-14 10:44:55   수정일: 2021-05-29 15:39:40 &lt;/Document-Metadata&gt;  === E…
+19. 2020년도_2020년 지사 맞춤형 사회적가치 실현  추진 계획(안)) #39  ▸  &lt;Document-Metadata&gt;   제목: 일자리 창출 중장기 계획   작성자: KRA   마지막 수정자: KRA   작성일: 2017-09-12 12:21:29   수정일: 2020-03-15 17:49:55 &lt;/Document-Metadata&gt;  &lt;table b…
+20. 2024년도_2024년 청심환 간담회 시행 계획(안) #2  ▸  &lt;Document-Metadata&gt;   제목: □    작성자: KRA   마지막 수정자: KRA   작성일: 2023-07-13 17:49:14   수정일: 2024-07-20 15:25:58 &lt;/Document-Metadata&gt;  □ 주요내용    ○ 참석 임차인 …
 ... +39 more</t>
         </is>
       </c>
@@ -5337,8 +5337,8 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[7b891a6e2bfdb9a0] (not found in graph)
-[d4e8e7e0de0bee24] (not found in graph)</t>
+          <t>1. [7b891a6e2bfdb9a0] (not found)
+2. [d4e8e7e0de0bee24] (not found)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -5372,8 +5372,8 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[abf6b885cc56106c] (not found in graph)
-[1d7a8c5b7cde9f12] (not found in graph)</t>
+          <t>1. [abf6b885cc56106c] (not found)
+2. [1d7a8c5b7cde9f12] (not found)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[a3e51e3ccd5f7a45] (not found in graph)</t>
+          <t>1. [a3e51e3ccd5f7a45] (not found)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[b5c2f8e7a11b3290] (not found in graph)</t>
+          <t>1. [b5c2f8e7a11b3290] (not found)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[e2b4c1d7f5a3a908] (not found in graph)</t>
+          <t>1. [e2b4c1d7f5a3a908] (not found)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -5506,8 +5506,8 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[f6a42e8c3b1d2f47] (not found in graph)
-[9c3e7a1b5d6f8290] (not found in graph)</t>
+          <t>1. [f6a42e8c3b1d2f47] (not found)
+2. [9c3e7a1b5d6f8290] (not found)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[c8f4e2d1a7b5c390] (not found in graph)</t>
+          <t>1. [c8f4e2d1a7b5c390] (not found)</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[a1b2c3d4e5f67890] (not found in graph)</t>
+          <t>1. [a1b2c3d4e5f67890] (not found)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[d7e9f1a3b5c79024] (not found in graph)</t>
+          <t>1. [d7e9f1a3b5c79024] (not found)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[b8c2d4e6f8a1b024] (not found in graph)</t>
+          <t>1. [b8c2d4e6f8a1b024] (not found)</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -5836,7 +5836,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00005] pr_goods_base:G00005  ▸  pr_goods_base: Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00003] pr_goods_base:G00003  ▸  pr_goods_base: Galaxy Book | 노트북 | G00003 | 2024-12-19 | Y | 150.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Galaxy Book | 노트북 | G00003 | 2024-12-19 | Y | 150.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00001] pr_goods_base:G00001  ▸  pr_goods_base: Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0</t>
+          <t>1. Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00002] pr_goods_base:G00002  ▸  pr_goods_base: CLA Mask | 일회용 마스크 | G00002 | 2024-12-19 | Y | 200.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0</t>
+          <t>1. CLA Mask | 일회용 마스크 | G00002 | 2024-12-19 | Y | 200.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00006] pr_goods_base:G00006  ▸  pr_goods_base: Volume Lip plumper maxi | 립밤 | G00006 | 2024-12-19 | Y | 200.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-</t>
+          <t>1. Volume Lip plumper maxi | 립밤 | G00006 | 2024-12-19 | Y | 200.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G01006] pr_goods_base:G01006  ▸  pr_goods_base: Cheese - Boursin, Garlic / Herbs | G01006 | 2023-12-18 | Y | 9999.0 | 77000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. Cheese - Boursin, Garlic / Herbs | G01006 | 2023-12-18 | Y | 9999.0 | 77000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -6034,8 +6034,8 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00010] pr_goods_base:G00010  ▸  pr_goods_base: Wine - Niagara,vqa Reisling | A | G00010 | 2023-12-18 | Y | 9999.0 | 78000.0 | 2023-12-19 00:00:00 | 2024
-[pr_goods_base:G00462] pr_goods_base:G00462  ▸  pr_goods_base: Wine - Niagara Peninsula Vqa | G00462 | 2023-12-18 | Y | 9999.0 | 22000.0 | 2023-12-19 00:00:00 | 2024-12</t>
+          <t>1. Wine - Niagara,vqa Reisling | A | G00010 | 2023-12-18 | Y | 9999.0 | 78000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Wine - Niagara Peninsula Vqa | G00462 | 2023-12-18 | Y | 9999.0 | 22000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -6069,7 +6069,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G01004] pr_goods_base:G01004  ▸  pr_goods_base: Chicken - Soup Base | G01004 | 2023-12-18 | Y | 9999.0 | 52000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00</t>
+          <t>1. Chicken - Soup Base | G01004 | 2023-12-18 | Y | 9999.0 | 52000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00992] pr_goods_base:G00992  ▸  pr_goods_base: Pastry - Banana Muffin - Mini | G00992 | 2023-12-18 | Y | 9999.0 | 24000.0 | 2023-12-19 00:00:00 | 2024-1</t>
+          <t>1. Pastry - Banana Muffin - Mini | G00992 | 2023-12-18 | Y | 9999.0 | 24000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -6135,8 +6135,8 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00082] pr_goods_base:G00082  ▸  pr_goods_base: Jameson - Irish Whiskey | G00082 | 2023-12-18 | Y | 9999.0 | 58000.0 | 2023-12-19 00:00:00 | 2024-12-18 0
-[pr_goods_base:G00968] pr_goods_base:G00968  ▸  pr_goods_base: Jameson Irish Whiskey | G00968 | 2023-12-18 | Y | 9999.0 | 15000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:</t>
+          <t>1. Jameson - Irish Whiskey | G00082 | 2023-12-18 | Y | 9999.0 | 58000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Jameson Irish Whiskey | G00968 | 2023-12-18 | Y | 9999.0 | 15000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -6170,8 +6170,8 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00470] pr_goods_base:G00470  ▸  pr_goods_base: Lamb Shoulder Boneless Nz | G00470 | 2023-12-18 | Y | 9999.0 | 61000.0 | 2023-12-19 00:00:00 | 2024-12-18
-[pr_goods_base:G00736] pr_goods_base:G00736  ▸  pr_goods_base: Lamb - Shoulder, Boneless | G00736 | 2023-12-18 | Y | 9999.0 | 25000.0 | 2023-12-19 00:00:00 | 2024-12-18</t>
+          <t>1. Lamb Shoulder Boneless Nz | G00470 | 2023-12-18 | Y | 9999.0 | 61000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Lamb - Shoulder, Boneless | G00736 | 2023-12-18 | Y | 9999.0 | 25000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -6205,8 +6205,8 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00467] pr_goods_base:G00467  ▸  pr_goods_base: English Muffin | G00467 | 2023-12-18 | Y | 9999.0 | 97000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |
-[pr_goods_base:G00569] pr_goods_base:G00569  ▸  pr_goods_base: English Muffin | G00569 | 2023-12-18 | Y | 9999.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |</t>
+          <t>1. English Muffin | G00467 | 2023-12-18 | Y | 9999.0 | 97000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. English Muffin | G00569 | 2023-12-18 | Y | 9999.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00974] pr_goods_base:G00974  ▸  pr_goods_base: Beer - Alexander Kieths, Pale Ale | G00974 | 2023-12-18 | Y | 9999.0 | 31000.0 | 2023-12-19 00:00:00 | 20</t>
+          <t>1. Beer - Alexander Kieths, Pale Ale | G00974 | 2023-12-18 | Y | 9999.0 | 31000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -6273,7 +6273,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00751] pr_goods_base:G00751  ▸  pr_goods_base: Wiberg Super Cure | G00751 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0</t>
+          <t>1. Wiberg Super Cure | G00751 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -6306,8 +6306,8 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00106] pr_goods_base:G00106  ▸  pr_goods_base: Wine - Ice Wine | G00106 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00339] pr_goods_base:G00339  ▸  pr_goods_base: Wine - Ice Wine | G00339 | 2023-12-18 | Y | 9999.0 | 39000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Wine - Ice Wine | G00106 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Wine - Ice Wine | G00339 | 2023-12-18 | Y | 9999.0 | 39000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -6341,8 +6341,8 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00315] pr_goods_base:G00315  ▸  pr_goods_base: Cheese - Feta | G00315 | 2023-12-18 | Y | 9999.0 | 97000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |
-[pr_goods_base:G00694] pr_goods_base:G00694  ▸  pr_goods_base: Cheese - Feta | G00694 | 2023-12-18 | Y | 9999.0 | 55000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |</t>
+          <t>1. Cheese - Feta | G00315 | 2023-12-18 | Y | 9999.0 | 97000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Cheese - Feta | G00694 | 2023-12-18 | Y | 9999.0 | 55000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00113] pr_goods_base:G00113  ▸  pr_goods_base: Wine - Cabernet Sauvignon | G00113 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18</t>
+          <t>1. Wine - Cabernet Sauvignon | G00113 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -6409,9 +6409,9 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00563] pr_goods_base:G00563  ▸  pr_goods_base: Bread - 10 Grain | G00563 | 2023-12-18 | Y | 9999.0 | 90000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00817] pr_goods_base:G00817  ▸  pr_goods_base: Bread - 10 Grain | G00817 | 2023-12-18 | Y | 9999.0 | 42000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G01005] pr_goods_base:G01005  ▸  pr_goods_base: Bread - 10 Grain | G01005 | 2023-12-18 | Y | 9999.0 | 17000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Bread - 10 Grain | G00563 | 2023-12-18 | Y | 9999.0 | 90000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Bread - 10 Grain | G00817 | 2023-12-18 | Y | 9999.0 | 42000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Bread - 10 Grain | G01005 | 2023-12-18 | Y | 9999.0 | 17000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00711] pr_goods_base:G00711  ▸  pr_goods_base: Garlic Powder | G00711 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2</t>
+          <t>1. Garlic Powder | G00711 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00005] pr_goods_base:G00005  ▸  pr_goods_base: Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -6699,10 +6699,10 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00040] pr_goods_base:G00040  ▸  pr_goods_base: Cheese - Provolone | G00040 | 2023-12-18 | Y | 9999.0 | 56000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:
-[pr_goods_base:G00083] pr_goods_base:G00083  ▸  pr_goods_base: Cheese - Gorgonzola | G00083 | 2023-12-18 | Y | 9999.0 | 26000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00
-[pr_goods_base:G00442] pr_goods_base:G00442  ▸  pr_goods_base: Cheese - Parmesan Cubes | G00442 | 2023-12-18 | Y | 9999.0 | 14000.0 | 2023-12-19 00:00:00 | 2024-12-18 0
-[pr_goods_base:G00158] pr_goods_base:G00158  ▸  pr_goods_base: Cheese - Mozzarella | G00158 | 2023-12-18 | Y | 9999.0 | 18000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00</t>
+          <t>1. Cheese - Provolone | G00040 | 2023-12-18 | Y | 9999.0 | 56000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Cheese - Gorgonzola | G00083 | 2023-12-18 | Y | 9999.0 | 26000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Cheese - Parmesan Cubes | G00442 | 2023-12-18 | Y | 9999.0 | 14000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Cheese - Mozzarella | G00158 | 2023-12-18 | Y | 9999.0 | 18000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00003] pr_goods_base:G00003  ▸  pr_goods_base: Galaxy Book | 노트북 | G00003 | 2024-12-19 | Y | 150.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Galaxy Book | 노트북 | G00003 | 2024-12-19 | Y | 150.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00001] pr_goods_base:G00001  ▸  pr_goods_base: Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0</t>
+          <t>1. Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00997] pr_goods_base:G00997  ▸  pr_goods_base: Cheese - Pont Couvert | G00997 | 2023-12-18 | Y | 9999.0 | 66000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:</t>
+          <t>1. Cheese - Pont Couvert | G00997 | 2023-12-18 | Y | 9999.0 | 66000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -6869,7 +6869,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -6951,10 +6951,10 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00072] pr_goods_base:G00072  ▸  pr_goods_base: Veal - Striploin | G00072 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00302] pr_goods_base:G00302  ▸  pr_goods_base: Oil - Olive | G00302 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 202
-[pr_goods_base:G00711] pr_goods_base:G00711  ▸  pr_goods_base: Garlic Powder | G00711 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2
-[pr_goods_base:G00892] pr_goods_base:G00892  ▸  pr_goods_base: Plate Pie Foil | G00892 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |</t>
+          <t>1. Veal - Striploin | G00072 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Oil - Olive | G00302 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Garlic Powder | G00711 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Plate Pie Foil | G00892 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -6998,26 +6998,26 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00005] pr_goods_base:G00005  ▸  pr_goods_base: Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00063] pr_goods_base:G00063  ▸  pr_goods_base: Chips Potato Swt Chilli Sour | G00063 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00068] pr_goods_base:G00068  ▸  pr_goods_base: Amarula Cream | G00068 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2
-[pr_goods_base:G00072] pr_goods_base:G00072  ▸  pr_goods_base: Veal - Striploin | G00072 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00089] pr_goods_base:G00089  ▸  pr_goods_base: Quail - Jumbo | G00089 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2
-[pr_goods_base:G00098] pr_goods_base:G00098  ▸  pr_goods_base: Fudge - Chocolate Fudge | G00098 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00
-[pr_goods_base:G00202] pr_goods_base:G00202  ▸  pr_goods_base: Pepper - Green Thai | G00202 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:
-[pr_goods_base:G00203] pr_goods_base:G00203  ▸  pr_goods_base: Jam - Raspberry,jar | G00203 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:
-[pr_goods_base:G00204] pr_goods_base:G00204  ▸  pr_goods_base: Oysters - Smoked | G00204 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00217] pr_goods_base:G00217  ▸  pr_goods_base: Soda Water - Club Soda, 355 Ml | G00217 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00258] pr_goods_base:G00258  ▸  pr_goods_base: Juice - Apple Cider | G00258 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:
-[pr_goods_base:G00261] pr_goods_base:G00261  ▸  pr_goods_base: Scotch - Queen Anne | G00261 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:
-[pr_goods_base:G00267] pr_goods_base:G00267  ▸  pr_goods_base: Soup - Campbells - Tomato | G00267 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18
-[pr_goods_base:G00283] pr_goods_base:G00283  ▸  pr_goods_base: Chinese Foods - Chicken Wing | G00283 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00302] pr_goods_base:G00302  ▸  pr_goods_base: Oil - Olive | G00302 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 202
-[pr_goods_base:G00314] pr_goods_base:G00314  ▸  pr_goods_base: Fondant - Icing | G00314 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |
-[pr_goods_base:G00332] pr_goods_base:G00332  ▸  pr_goods_base: Nut - Walnut, Chopped | G00332 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:0
-[pr_goods_base:G00376] pr_goods_base:G00376  ▸  pr_goods_base: Otomegusa Dashi Konbu | G00376 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:0
-[pr_goods_base:G00388] pr_goods_base:G00388  ▸  pr_goods_base: Lettuce - Iceberg | G00388 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00438] pr_goods_base:G00438  ▸  pr_goods_base: Doilies - 8, Paper | G00438 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0
+          <t>1. Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Chips Potato Swt Chilli Sour | G00063 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Amarula Cream | G00068 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Veal - Striploin | G00072 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+5. Quail - Jumbo | G00089 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+6. Fudge - Chocolate Fudge | G00098 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+7. Pepper - Green Thai | G00202 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+8. Jam - Raspberry,jar | G00203 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+9. Oysters - Smoked | G00204 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+10. Soda Water - Club Soda, 355 Ml | G00217 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+11. Juice - Apple Cider | G00258 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+12. Scotch - Queen Anne | G00261 | 2023-12-18 | Y | 9999.0 | 3000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+13. Soup - Campbells - Tomato | G00267 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+14. Chinese Foods - Chicken Wing | G00283 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+15. Oil - Olive | G00302 | 2023-12-18 | Y | 9999.0 | 1000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+16. Fondant - Icing | G00314 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+17. Nut - Walnut, Chopped | G00332 | 2023-12-18 | Y | 9999.0 | 4000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+18. Otomegusa Dashi Konbu | G00376 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+19. Lettuce - Iceberg | G00388 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+20. Doilies - 8, Paper | G00438 | 2023-12-18 | Y | 9999.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
 ... +21 more</t>
         </is>
       </c>
@@ -7099,9 +7099,9 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00001] pr_goods_base:G00001  ▸  pr_goods_base: Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0
-[pr_goods_base:G00004] pr_goods_base:G00004  ▸  pr_goods_base: Jacket | 남성 의류 | G00004 | 2024-12-19 | Y | 200.0 | 18500.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 |
-[pr_goods_base:G00007] pr_goods_base:G00007  ▸  pr_goods_base: iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 202</t>
+          <t>1. Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Jacket | 남성 의류 | G00004 | 2024-12-19 | Y | 200.0 | 18500.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. iPhone 15 Pro 512GB | 아이폰 15 프로 | G00007 | 2024-12-19 | Y | 200.0 | 1600000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -7144,11 +7144,11 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00751] pr_goods_base:G00751  ▸  pr_goods_base: Wiberg Super Cure | G00751 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0
-[pr_goods_base:G00472] pr_goods_base:G00472  ▸  pr_goods_base: Bread - Kimel Stick Poly | G00472 | 2023-12-18 | Y | 9999.0 | 42000.0 | 2023-12-19 00:00:00 | 2024-12-18
-[pr_goods_base:G00389] pr_goods_base:G00389  ▸  pr_goods_base: Pork Ham Prager | G00389 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00329] pr_goods_base:G00329  ▸  pr_goods_base: Sauce - Ranch Dressing | G00329 | 2023-12-18 | Y | 9999.0 | 88000.0 | 2023-12-19 00:00:00 | 2024-12-18 00
-[pr_goods_base:G00997] pr_goods_base:G00997  ▸  pr_goods_base: Cheese - Pont Couvert | G00997 | 2023-12-18 | Y | 9999.0 | 66000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:</t>
+          <t>1. Wiberg Super Cure | G00751 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Bread - Kimel Stick Poly | G00472 | 2023-12-18 | Y | 9999.0 | 42000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Pork Ham Prager | G00389 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Sauce - Ranch Dressing | G00329 | 2023-12-18 | Y | 9999.0 | 88000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+5. Cheese - Pont Couvert | G00997 | 2023-12-18 | Y | 9999.0 | 66000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -7193,17 +7193,17 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00270] pr_goods_base:G00270  ▸  pr_goods_base: Beer - Mill St Organic | G00270 | 2023-12-18 | Y | 9999.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00
-[pr_goods_base:G00466] pr_goods_base:G00466  ▸  pr_goods_base: Beer - Sleemans Honey Brown | G00466 | 2023-12-18 | Y | 9999.0 | 47000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00645] pr_goods_base:G00645  ▸  pr_goods_base: Beer - Original Organic Lager | G00645 | 2023-12-18 | Y | 9999.0 | 73000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00700] pr_goods_base:G00700  ▸  pr_goods_base: Beer - Moosehead | G00700 | 2023-12-18 | Y | 9999.0 | 87000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00719] pr_goods_base:G00719  ▸  pr_goods_base: Beer - Original Organic Lager | G00719 | 2023-12-18 | Y | 9999.0 | 74000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00793] pr_goods_base:G00793  ▸  pr_goods_base: Beer - Steamwhistle | G00793 | 2023-12-18 | Y | 9999.0 | 33000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00
-[pr_goods_base:G00798] pr_goods_base:G00798  ▸  pr_goods_base: Beer - Original Organic Lager | G00798 | 2023-12-18 | Y | 9999.0 | 90000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00928] pr_goods_base:G00928  ▸  pr_goods_base: Beer - Rickards Red | G00928 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00
-[pr_goods_base:G00937] pr_goods_base:G00937  ▸  pr_goods_base: Beer - Mcauslan Apricot | G00937 | 2023-12-18 | Y | 9999.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 0
-[pr_goods_base:G00938] pr_goods_base:G00938  ▸  pr_goods_base: Beer - Steamwhistle | G00938 | 2023-12-18 | Y | 9999.0 | 63000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00
-[pr_goods_base:G00974] pr_goods_base:G00974  ▸  pr_goods_base: Beer - Alexander Kieths, Pale Ale | G00974 | 2023-12-18 | Y | 9999.0 | 31000.0 | 2023-12-19 00:00:00 | 20</t>
+          <t>1. Beer - Mill St Organic | G00270 | 2023-12-18 | Y | 9999.0 | 59000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Beer - Sleemans Honey Brown | G00466 | 2023-12-18 | Y | 9999.0 | 47000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Beer - Original Organic Lager | G00645 | 2023-12-18 | Y | 9999.0 | 73000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Beer - Moosehead | G00700 | 2023-12-18 | Y | 9999.0 | 87000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+5. Beer - Original Organic Lager | G00719 | 2023-12-18 | Y | 9999.0 | 74000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+6. Beer - Steamwhistle | G00793 | 2023-12-18 | Y | 9999.0 | 33000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+7. Beer - Original Organic Lager | G00798 | 2023-12-18 | Y | 9999.0 | 90000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+8. Beer - Rickards Red | G00928 | 2023-12-18 | Y | 9999.0 | 36000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+9. Beer - Mcauslan Apricot | G00937 | 2023-12-18 | Y | 9999.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+10. Beer - Steamwhistle | G00938 | 2023-12-18 | Y | 9999.0 | 63000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+11. Beer - Alexander Kieths, Pale Ale | G00974 | 2023-12-18 | Y | 9999.0 | 31000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00857] pr_goods_base:G00857  ▸  pr_goods_base: Flour - Masa De Harina Mexican | G00857 | 2023-12-18 | Y | 9999.0 | 86000.0 | 2023-12-19 00:00:00 | 2024-</t>
+          <t>1. Flour - Masa De Harina Mexican | G00857 | 2023-12-18 | Y | 9999.0 | 86000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00001] pr_goods_base:G00001  ▸  pr_goods_base: Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0</t>
+          <t>1. Dried Beef | 소고기육포 | G00001 | 2024-12-19 | Y | 100.0 | 40000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -7336,26 +7336,26 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00010] pr_goods_base:G00010  ▸  pr_goods_base: Wine - Niagara,vqa Reisling | A | G00010 | 2023-12-18 | Y | 9999.0 | 78000.0 | 2023-12-19 00:00:00 | 2024
-[pr_goods_base:G00034] pr_goods_base:G00034  ▸  pr_goods_base: Wine - Piper Heidsieck Brut | G00034 | 2023-12-18 | Y | 9999.0 | 47000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00048] pr_goods_base:G00048  ▸  pr_goods_base: Wine - Sicilia Igt Nero Avola | G00048 | 2023-12-18 | Y | 9999.0 | 18000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00055] pr_goods_base:G00055  ▸  pr_goods_base: Wine - Champagne Brut Veuve | G00055 | 2023-12-18 | Y | 9999.0 | 10000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00077] pr_goods_base:G00077  ▸  pr_goods_base: Wine - Magnotta, White | G00077 | 2023-12-18 | Y | 9999.0 | 26000.0 | 2023-12-19 00:00:00 | 2024-12-18 00
-[pr_goods_base:G00086] pr_goods_base:G00086  ▸  pr_goods_base: Wine - Winzer Krems Gruner | G00086 | 2023-12-18 | Y | 9999.0 | 75000.0 | 2023-12-19 00:00:00 | 2024-12-1
-[pr_goods_base:G00106] pr_goods_base:G00106  ▸  pr_goods_base: Wine - Ice Wine | G00106 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00112] pr_goods_base:G00112  ▸  pr_goods_base: Wine - Red, Cabernet Merlot | G00112 | 2023-12-18 | Y | 9999.0 | 14000.0 | 2023-12-19 00:00:00 | 2024-12-
-[pr_goods_base:G00113] pr_goods_base:G00113  ▸  pr_goods_base: Wine - Cabernet Sauvignon | G00113 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18
-[pr_goods_base:G00138] pr_goods_base:G00138  ▸  pr_goods_base: Wine - Fino Tio Pepe Gonzalez | G00138 | 2023-12-18 | Y | 9999.0 | 64000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00144] pr_goods_base:G00144  ▸  pr_goods_base: Wine - Tribal Sauvignon | G00144 | 2023-12-18 | Y | 9999.0 | 38000.0 | 2023-12-19 00:00:00 | 2024-12-18 0
-[pr_goods_base:G00148] pr_goods_base:G00148  ▸  pr_goods_base: Wine - Delicato Merlot | G00148 | 2023-12-18 | Y | 9999.0 | 17000.0 | 2023-12-19 00:00:00 | 2024-12-18 00
-[pr_goods_base:G00164] pr_goods_base:G00164  ▸  pr_goods_base: Wine - Pinot Grigio Collavini | G00164 | 2023-12-18 | Y | 9999.0 | 65000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00172] pr_goods_base:G00172  ▸  pr_goods_base: Wine - Red, Pinot Noir, Chateau | G00172 | 2023-12-18 | Y | 9999.0 | 48000.0 | 2023-12-19 00:00:00 | 2024
-[pr_goods_base:G00174] pr_goods_base:G00174  ▸  pr_goods_base: Wine La Vielle Ferme Cote Du | G00174 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12
-[pr_goods_base:G00207] pr_goods_base:G00207  ▸  pr_goods_base: Wine - Rubyport | G00207 | 2023-12-18 | Y | 9999.0 | 65000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00
-[pr_goods_base:G00264] pr_goods_base:G00264  ▸  pr_goods_base: Wine - Rosso Del Veronese Igt | G00264 | 2023-12-18 | Y | 9999.0 | 54000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00277] pr_goods_base:G00277  ▸  pr_goods_base: Wine - Wyndham Estate Bin 777 | G00277 | 2023-12-18 | Y | 9999.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00282] pr_goods_base:G00282  ▸  pr_goods_base: Wine - Chateauneuf Du Pape | G00282 | 2023-12-18 | Y | 9999.0 | 29000.0 | 2023-12-19 00:00:00 | 2024-12-1
-[pr_goods_base:G00293] pr_goods_base:G00293  ▸  pr_goods_base: Wine - Casablanca Valley | G00293 | 2023-12-18 | Y | 9999.0 | 12000.0 | 2023-12-19 00:00:00 | 2024-12-18
+          <t>1. Wine - Niagara,vqa Reisling | A | G00010 | 2023-12-18 | Y | 9999.0 | 78000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Wine - Piper Heidsieck Brut | G00034 | 2023-12-18 | Y | 9999.0 | 47000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Wine - Sicilia Igt Nero Avola | G00048 | 2023-12-18 | Y | 9999.0 | 18000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+4. Wine - Champagne Brut Veuve | G00055 | 2023-12-18 | Y | 9999.0 | 10000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+5. Wine - Magnotta, White | G00077 | 2023-12-18 | Y | 9999.0 | 26000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+6. Wine - Winzer Krems Gruner | G00086 | 2023-12-18 | Y | 9999.0 | 75000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+7. Wine - Ice Wine | G00106 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+8. Wine - Red, Cabernet Merlot | G00112 | 2023-12-18 | Y | 9999.0 | 14000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+9. Wine - Cabernet Sauvignon | G00113 | 2023-12-18 | Y | 9999.0 | 41000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+10. Wine - Fino Tio Pepe Gonzalez | G00138 | 2023-12-18 | Y | 9999.0 | 64000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+11. Wine - Tribal Sauvignon | G00144 | 2023-12-18 | Y | 9999.0 | 38000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+12. Wine - Delicato Merlot | G00148 | 2023-12-18 | Y | 9999.0 | 17000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+13. Wine - Pinot Grigio Collavini | G00164 | 2023-12-18 | Y | 9999.0 | 65000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+14. Wine - Red, Pinot Noir, Chateau | G00172 | 2023-12-18 | Y | 9999.0 | 48000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+15. Wine La Vielle Ferme Cote Du | G00174 | 2023-12-18 | Y | 9999.0 | 85000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+16. Wine - Rubyport | G00207 | 2023-12-18 | Y | 9999.0 | 65000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+17. Wine - Rosso Del Veronese Igt | G00264 | 2023-12-18 | Y | 9999.0 | 54000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+18. Wine - Wyndham Estate Bin 777 | G00277 | 2023-12-18 | Y | 9999.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+19. Wine - Chateauneuf Du Pape | G00282 | 2023-12-18 | Y | 9999.0 | 29000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+20. Wine - Casablanca Valley | G00293 | 2023-12-18 | Y | 9999.0 | 12000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
 ... +10 more</t>
         </is>
       </c>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00005] pr_goods_base:G00005  ▸  pr_goods_base: Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00</t>
+          <t>1. Shin Ramyun | 신라면 | G00005 | 2024-12-19 | Y | 150.0 | 5000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -7467,9 +7467,9 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00470] pr_goods_base:G00470  ▸  pr_goods_base: Lamb Shoulder Boneless Nz | G00470 | 2023-12-18 | Y | 9999.0 | 61000.0 | 2023-12-19 00:00:00 | 2024-12-18
-[pr_goods_base:G00492] pr_goods_base:G00492  ▸  pr_goods_base: Lamb - Loin, Trimmed, Boneless | G00492 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-1
-[pr_goods_base:G00736] pr_goods_base:G00736  ▸  pr_goods_base: Lamb - Shoulder, Boneless | G00736 | 2023-12-18 | Y | 9999.0 | 25000.0 | 2023-12-19 00:00:00 | 2024-12-18</t>
+          <t>1. Lamb Shoulder Boneless Nz | G00470 | 2023-12-18 | Y | 9999.0 | 61000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Lamb - Loin, Trimmed, Boneless | G00492 | 2023-12-18 | Y | 9999.0 | 2000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+3. Lamb - Shoulder, Boneless | G00736 | 2023-12-18 | Y | 9999.0 | 25000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -7512,8 +7512,8 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>[pr_goods_base:G00002] pr_goods_base:G00002  ▸  pr_goods_base: CLA Mask | 일회용 마스크 | G00002 | 2024-12-19 | Y | 200.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:0
-[pr_goods_base:G00006] pr_goods_base:G00006  ▸  pr_goods_base: Volume Lip plumper maxi | 립밤 | G00006 | 2024-12-19 | Y | 200.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-</t>
+          <t>1. CLA Mask | 일회용 마스크 | G00002 | 2024-12-19 | Y | 200.0 | 72000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00
+2. Volume Lip plumper maxi | 립밤 | G00006 | 2024-12-19 | Y | 200.0 | 16000.0 | 2023-12-19 00:00:00 | 2024-12-18 00:00:00 | 2023-12-19 00:00:00</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">

</xml_diff>